<commit_message>
Adiciona linha TOTAL (65) na tabela DCMD por responsável da Visão ETO
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBtNB8AfUGxQoc5b1rirVp
</commit_message>
<xml_diff>
--- a/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
+++ b/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -315,6 +315,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2619,7 +2628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2841,2992 +2850,3008 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="56" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>21</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="56" t="inlineStr">
         <is>
           <t>Definições do gestor (08/07): 5850308009 (Guaraí) = NÃO concluído — segue no posto do COEP/fila DCMD; 7942572059 (Taquaralto) = melhoria de aterramento SEM CUSTO, considerado EM EXECUÇÃO via ETO-RD-PA 00427/2026 (SS ainda aberta).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Lista oficial DCMD (ETO 36) — 65 equipamentos</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>SS SGM</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Criticidade (oficial)</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Dias aguardando DCMD</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Dias pendente (SS)</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Responsável</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Município</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Está no orçamento?</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>Situação no mapeamento</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="57" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="62" t="inlineStr">
         <is>
           <t>7923927122</t>
         </is>
       </c>
-      <c r="B23" s="57" t="inlineStr">
+      <c r="B24" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C23" s="58" t="inlineStr">
+      <c r="C24" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00079/2025</t>
         </is>
       </c>
-      <c r="D23" s="57" t="inlineStr">
+      <c r="D24" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E23" s="57" t="n">
+      <c r="E24" s="62" t="n">
         <v>434</v>
       </c>
-      <c r="G23" s="57" t="inlineStr">
+      <c r="G24" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H23" s="58" t="inlineStr">
+      <c r="H24" s="63" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I23" s="58" t="inlineStr">
+      <c r="I24" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J23" s="23" t="inlineStr">
+      <c r="J24" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="57" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="62" t="inlineStr">
         <is>
           <t>7900532053</t>
         </is>
       </c>
-      <c r="B24" s="57" t="inlineStr">
+      <c r="B25" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C24" s="58" t="inlineStr">
+      <c r="C25" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00102/2025</t>
         </is>
       </c>
-      <c r="D24" s="57" t="inlineStr">
+      <c r="D25" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E24" s="57" t="n">
+      <c r="E25" s="62" t="n">
         <v>407</v>
       </c>
-      <c r="G24" s="57" t="inlineStr">
+      <c r="G25" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H24" s="58" t="inlineStr">
+      <c r="H25" s="63" t="inlineStr">
         <is>
           <t>Piraque</t>
         </is>
       </c>
-      <c r="I24" s="58" t="inlineStr">
+      <c r="I25" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J24" s="23" t="inlineStr">
+      <c r="J25" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="57" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="62" t="inlineStr">
         <is>
           <t>7920024127</t>
         </is>
       </c>
-      <c r="B25" s="57" t="inlineStr">
+      <c r="B26" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C25" s="58" t="inlineStr">
+      <c r="C26" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00120/2025</t>
         </is>
       </c>
-      <c r="D25" s="57" t="inlineStr">
+      <c r="D26" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E25" s="57" t="n">
+      <c r="E26" s="62" t="n">
         <v>371</v>
       </c>
-      <c r="G25" s="57" t="inlineStr">
+      <c r="G26" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H25" s="58" t="inlineStr">
+      <c r="H26" s="63" t="inlineStr">
         <is>
           <t>Palmeiras Do Tocantins</t>
         </is>
       </c>
-      <c r="I25" s="58" t="inlineStr">
+      <c r="I26" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J25" s="23" t="inlineStr">
+      <c r="J26" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="57" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="62" t="inlineStr">
         <is>
           <t>5858783119</t>
         </is>
       </c>
-      <c r="B26" s="57" t="inlineStr">
+      <c r="B27" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C26" s="58" t="inlineStr">
+      <c r="C27" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00123/2025</t>
         </is>
       </c>
-      <c r="D26" s="57" t="inlineStr">
+      <c r="D27" s="62" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E26" s="57" t="n">
+      <c r="E27" s="62" t="n">
         <v>369</v>
       </c>
-      <c r="G26" s="57" t="inlineStr">
+      <c r="G27" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H26" s="58" t="inlineStr">
+      <c r="H27" s="63" t="inlineStr">
         <is>
           <t>Sao Bento Do Tocantins</t>
         </is>
       </c>
-      <c r="I26" s="58" t="inlineStr">
+      <c r="I27" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J26" s="23" t="inlineStr">
+      <c r="J27" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="57" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="62" t="inlineStr">
         <is>
           <t>7927446001</t>
         </is>
       </c>
-      <c r="B27" s="57" t="inlineStr">
+      <c r="B28" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C27" s="58" t="inlineStr">
+      <c r="C28" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00143/2025</t>
         </is>
       </c>
-      <c r="D27" s="57" t="inlineStr">
+      <c r="D28" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E27" s="57" t="n">
+      <c r="E28" s="62" t="n">
         <v>364</v>
       </c>
-      <c r="G27" s="57" t="inlineStr">
+      <c r="G28" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H27" s="58" t="inlineStr">
+      <c r="H28" s="63" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I27" s="58" t="inlineStr">
+      <c r="I28" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J27" s="23" t="inlineStr">
+      <c r="J28" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="57" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="62" t="inlineStr">
         <is>
           <t>7957126085</t>
         </is>
       </c>
-      <c r="B28" s="57" t="inlineStr">
+      <c r="B29" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C28" s="58" t="inlineStr">
+      <c r="C29" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00156/2025</t>
         </is>
       </c>
-      <c r="D28" s="57" t="inlineStr">
+      <c r="D29" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E28" s="57" t="n">
+      <c r="E29" s="62" t="n">
         <v>350</v>
       </c>
-      <c r="G28" s="57" t="inlineStr">
+      <c r="G29" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H28" s="58" t="inlineStr">
+      <c r="H29" s="63" t="inlineStr">
         <is>
           <t>Monte Santo Do Tocantins</t>
         </is>
       </c>
-      <c r="I28" s="58" t="inlineStr">
+      <c r="I29" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J28" s="23" t="inlineStr">
+      <c r="J29" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="57" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="62" t="inlineStr">
         <is>
           <t>7942485096</t>
         </is>
       </c>
-      <c r="B29" s="57" t="inlineStr">
+      <c r="B30" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C29" s="58" t="inlineStr">
+      <c r="C30" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00158/2025</t>
         </is>
       </c>
-      <c r="D29" s="57" t="inlineStr">
+      <c r="D30" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E29" s="57" t="n">
+      <c r="E30" s="62" t="n">
         <v>349</v>
       </c>
-      <c r="G29" s="57" t="inlineStr">
+      <c r="G30" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H29" s="58" t="inlineStr">
+      <c r="H30" s="63" t="inlineStr">
         <is>
           <t>Pindorama Do Tocantins</t>
         </is>
       </c>
-      <c r="I29" s="58" t="inlineStr">
+      <c r="I30" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J29" s="23" t="inlineStr">
+      <c r="J30" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="57" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="62" t="inlineStr">
         <is>
           <t>5854566043</t>
         </is>
       </c>
-      <c r="B30" s="57" t="inlineStr">
+      <c r="B31" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C30" s="58" t="inlineStr">
+      <c r="C31" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00160/2025</t>
         </is>
       </c>
-      <c r="D30" s="57" t="inlineStr">
+      <c r="D31" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E30" s="57" t="n">
+      <c r="E31" s="62" t="n">
         <v>347</v>
       </c>
-      <c r="G30" s="57" t="inlineStr">
+      <c r="G31" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H30" s="58" t="inlineStr">
+      <c r="H31" s="63" t="inlineStr">
         <is>
           <t>Silvanopolis</t>
         </is>
       </c>
-      <c r="I30" s="58" t="inlineStr">
+      <c r="I31" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J30" s="23" t="inlineStr">
+      <c r="J31" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="57" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="62" t="inlineStr">
         <is>
           <t>5844630060</t>
         </is>
       </c>
-      <c r="B31" s="57" t="inlineStr">
+      <c r="B32" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C31" s="58" t="inlineStr">
+      <c r="C32" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00167/2025</t>
         </is>
       </c>
-      <c r="D31" s="57" t="inlineStr">
+      <c r="D32" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E31" s="57" t="n">
+      <c r="E32" s="62" t="n">
         <v>333</v>
       </c>
-      <c r="G31" s="57" t="inlineStr">
+      <c r="G32" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H31" s="58" t="inlineStr">
+      <c r="H32" s="63" t="inlineStr">
         <is>
           <t>Nova Olinda</t>
         </is>
       </c>
-      <c r="I31" s="58" t="inlineStr">
+      <c r="I32" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J31" s="23" t="inlineStr">
+      <c r="J32" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="57" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="62" t="inlineStr">
         <is>
           <t>7900535058</t>
         </is>
       </c>
-      <c r="B32" s="57" t="inlineStr">
+      <c r="B33" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C32" s="58" t="inlineStr">
+      <c r="C33" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00173/2025</t>
         </is>
       </c>
-      <c r="D32" s="57" t="inlineStr">
+      <c r="D33" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E32" s="57" t="n">
+      <c r="E33" s="62" t="n">
         <v>317</v>
       </c>
-      <c r="G32" s="57" t="inlineStr">
+      <c r="G33" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H32" s="58" t="inlineStr">
+      <c r="H33" s="63" t="inlineStr">
         <is>
           <t>Santa Fe Do Araguaia</t>
         </is>
       </c>
-      <c r="I32" s="58" t="inlineStr">
+      <c r="I33" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J32" s="23" t="inlineStr">
+      <c r="J33" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="57" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="62" t="inlineStr">
         <is>
           <t>7903112004</t>
         </is>
       </c>
-      <c r="B33" s="57" t="inlineStr">
+      <c r="B34" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C33" s="58" t="inlineStr">
+      <c r="C34" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00184/2025</t>
         </is>
       </c>
-      <c r="D33" s="57" t="inlineStr">
+      <c r="D34" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E33" s="57" t="n">
+      <c r="E34" s="62" t="n">
         <v>307</v>
       </c>
-      <c r="G33" s="57" t="inlineStr">
+      <c r="G34" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H33" s="58" t="inlineStr">
+      <c r="H34" s="63" t="inlineStr">
         <is>
           <t>Araguaina</t>
         </is>
       </c>
-      <c r="I33" s="58" t="inlineStr">
+      <c r="I34" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J33" s="23" t="inlineStr">
+      <c r="J34" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="57" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="62" t="inlineStr">
         <is>
           <t>5800371025</t>
         </is>
       </c>
-      <c r="B34" s="57" t="inlineStr">
+      <c r="B35" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C34" s="58" t="inlineStr">
+      <c r="C35" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00187/2025</t>
         </is>
       </c>
-      <c r="D34" s="57" t="inlineStr">
+      <c r="D35" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E34" s="57" t="n">
+      <c r="E35" s="62" t="n">
         <v>305</v>
       </c>
-      <c r="G34" s="57" t="inlineStr">
+      <c r="G35" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H34" s="58" t="inlineStr">
+      <c r="H35" s="63" t="inlineStr">
         <is>
           <t>Arapoema</t>
         </is>
       </c>
-      <c r="I34" s="58" t="inlineStr">
+      <c r="I35" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J34" s="23" t="inlineStr">
+      <c r="J35" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="57" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="62" t="inlineStr">
         <is>
           <t>5855411017</t>
         </is>
       </c>
-      <c r="B35" s="57" t="inlineStr">
+      <c r="B36" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C35" s="58" t="inlineStr">
+      <c r="C36" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00199/2025</t>
         </is>
       </c>
-      <c r="D35" s="57" t="inlineStr">
+      <c r="D36" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E35" s="57" t="n">
+      <c r="E36" s="62" t="n">
         <v>280</v>
       </c>
-      <c r="G35" s="57" t="inlineStr">
+      <c r="G36" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H35" s="58" t="inlineStr">
+      <c r="H36" s="63" t="inlineStr">
         <is>
           <t>Barrolandia</t>
         </is>
       </c>
-      <c r="I35" s="58" t="inlineStr">
+      <c r="I36" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J35" s="23" t="inlineStr">
+      <c r="J36" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="57" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="62" t="inlineStr">
         <is>
           <t>5853360007</t>
         </is>
       </c>
-      <c r="B36" s="57" t="inlineStr">
+      <c r="B37" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C36" s="58" t="inlineStr">
+      <c r="C37" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PS 00323/2025</t>
         </is>
       </c>
-      <c r="D36" s="57" t="inlineStr">
+      <c r="D37" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E36" s="57" t="n">
+      <c r="E37" s="62" t="n">
         <v>264</v>
       </c>
-      <c r="G36" s="57" t="inlineStr">
+      <c r="G37" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H36" s="58" t="inlineStr">
+      <c r="H37" s="63" t="inlineStr">
         <is>
           <t>Miracema Do Tocantins</t>
         </is>
       </c>
-      <c r="I36" s="59" t="inlineStr">
+      <c r="I37" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J36" s="23" t="inlineStr">
+      <c r="J37" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="57" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="62" t="inlineStr">
         <is>
           <t>5800961074</t>
         </is>
       </c>
-      <c r="B37" s="57" t="inlineStr">
+      <c r="B38" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C37" s="58" t="inlineStr">
+      <c r="C38" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00221/2025</t>
         </is>
       </c>
-      <c r="D37" s="57" t="inlineStr">
+      <c r="D38" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E37" s="57" t="n">
+      <c r="E38" s="62" t="n">
         <v>214</v>
       </c>
-      <c r="G37" s="57" t="inlineStr">
+      <c r="G38" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H37" s="58" t="inlineStr">
+      <c r="H38" s="63" t="inlineStr">
         <is>
           <t>Dianopolis</t>
         </is>
       </c>
-      <c r="I37" s="58" t="inlineStr">
+      <c r="I38" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J37" s="23" t="inlineStr">
+      <c r="J38" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="57" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="62" t="inlineStr">
         <is>
           <t>7925087021</t>
         </is>
       </c>
-      <c r="B38" s="57" t="inlineStr">
+      <c r="B39" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C38" s="58" t="inlineStr">
+      <c r="C39" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00222/2025</t>
         </is>
       </c>
-      <c r="D38" s="57" t="inlineStr">
+      <c r="D39" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E38" s="57" t="n">
+      <c r="E39" s="62" t="n">
         <v>211</v>
       </c>
-      <c r="G38" s="57" t="inlineStr">
+      <c r="G39" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H38" s="58" t="inlineStr">
+      <c r="H39" s="63" t="inlineStr">
         <is>
           <t>Parana</t>
         </is>
       </c>
-      <c r="I38" s="58" t="inlineStr">
+      <c r="I39" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J38" s="23" t="inlineStr">
+      <c r="J39" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="57" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="62" t="inlineStr">
         <is>
           <t>5862236091</t>
         </is>
       </c>
-      <c r="B39" s="57" t="inlineStr">
+      <c r="B40" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C39" s="58" t="inlineStr">
+      <c r="C40" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00223/2025</t>
         </is>
       </c>
-      <c r="D39" s="57" t="inlineStr">
+      <c r="D40" s="62" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E39" s="57" t="n">
+      <c r="E40" s="62" t="n">
         <v>211</v>
       </c>
-      <c r="G39" s="57" t="inlineStr">
+      <c r="G40" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H39" s="58" t="inlineStr">
+      <c r="H40" s="63" t="inlineStr">
         <is>
           <t>Almas</t>
         </is>
       </c>
-      <c r="I39" s="58" t="inlineStr">
+      <c r="I40" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J39" s="23" t="inlineStr">
+      <c r="J40" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="57" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="62" t="inlineStr">
         <is>
           <t>7933585074</t>
         </is>
       </c>
-      <c r="B40" s="57" t="inlineStr">
+      <c r="B41" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C40" s="58" t="inlineStr">
+      <c r="C41" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00024/2026</t>
         </is>
       </c>
-      <c r="D40" s="57" t="inlineStr">
+      <c r="D41" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E40" s="57" t="n">
+      <c r="E41" s="62" t="n">
         <v>161</v>
       </c>
-      <c r="G40" s="57" t="inlineStr">
+      <c r="G41" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H40" s="58" t="inlineStr">
+      <c r="H41" s="63" t="inlineStr">
         <is>
           <t>Dianopolis</t>
         </is>
       </c>
-      <c r="I40" s="58" t="inlineStr">
+      <c r="I41" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J40" s="23" t="inlineStr">
+      <c r="J41" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="57" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="62" t="inlineStr">
         <is>
           <t>7927646026</t>
         </is>
       </c>
-      <c r="B41" s="57" t="inlineStr">
+      <c r="B42" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C41" s="58" t="inlineStr">
+      <c r="C42" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00029/2026</t>
         </is>
       </c>
-      <c r="D41" s="57" t="inlineStr">
+      <c r="D42" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E41" s="57" t="n">
+      <c r="E42" s="62" t="n">
         <v>154</v>
       </c>
-      <c r="G41" s="57" t="inlineStr">
+      <c r="G42" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H41" s="58" t="inlineStr">
+      <c r="H42" s="63" t="inlineStr">
         <is>
           <t>Ponte Alta Tocantins</t>
         </is>
       </c>
-      <c r="I41" s="58" t="inlineStr">
+      <c r="I42" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J41" s="23" t="inlineStr">
+      <c r="J42" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="57" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="62" t="inlineStr">
         <is>
           <t>7931608059</t>
         </is>
       </c>
-      <c r="B42" s="57" t="inlineStr">
+      <c r="B43" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C42" s="58" t="inlineStr">
+      <c r="C43" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00040/2026</t>
         </is>
       </c>
-      <c r="D42" s="57" t="inlineStr">
+      <c r="D43" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E42" s="57" t="n">
+      <c r="E43" s="62" t="n">
         <v>133</v>
       </c>
-      <c r="G42" s="57" t="inlineStr">
+      <c r="G43" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H42" s="58" t="inlineStr">
+      <c r="H43" s="63" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I42" s="58" t="inlineStr">
+      <c r="I43" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J42" s="23" t="inlineStr">
+      <c r="J43" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="57" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="62" t="inlineStr">
         <is>
           <t>7908249152</t>
         </is>
       </c>
-      <c r="B43" s="57" t="inlineStr">
+      <c r="B44" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C43" s="58" t="inlineStr">
+      <c r="C44" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00038/2026</t>
         </is>
       </c>
-      <c r="D43" s="57" t="inlineStr">
+      <c r="D44" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E43" s="57" t="n">
+      <c r="E44" s="62" t="n">
         <v>133</v>
       </c>
-      <c r="G43" s="57" t="inlineStr">
+      <c r="G44" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H43" s="58" t="inlineStr">
+      <c r="H44" s="63" t="inlineStr">
         <is>
           <t>Santa Rosa Do Tocantins</t>
         </is>
       </c>
-      <c r="I43" s="58" t="inlineStr">
+      <c r="I44" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J43" s="23" t="inlineStr">
+      <c r="J44" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="57" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="62" t="inlineStr">
         <is>
           <t>7927396052</t>
         </is>
       </c>
-      <c r="B44" s="57" t="inlineStr">
+      <c r="B45" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C44" s="58" t="inlineStr">
+      <c r="C45" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00045/2026</t>
         </is>
       </c>
-      <c r="D44" s="57" t="inlineStr">
+      <c r="D45" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E44" s="57" t="n">
+      <c r="E45" s="62" t="n">
         <v>127</v>
       </c>
-      <c r="G44" s="57" t="inlineStr">
+      <c r="G45" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H44" s="58" t="inlineStr">
+      <c r="H45" s="63" t="inlineStr">
         <is>
           <t>Formoso Do Araguaia</t>
         </is>
       </c>
-      <c r="I44" s="58" t="inlineStr">
+      <c r="I45" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J44" s="23" t="inlineStr">
+      <c r="J45" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="57" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="62" t="inlineStr">
         <is>
           <t>7925871077</t>
         </is>
       </c>
-      <c r="B45" s="57" t="inlineStr">
+      <c r="B46" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C45" s="58" t="inlineStr">
+      <c r="C46" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00048/2026</t>
         </is>
       </c>
-      <c r="D45" s="57" t="inlineStr">
+      <c r="D46" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E45" s="57" t="n">
+      <c r="E46" s="62" t="n">
         <v>113</v>
       </c>
-      <c r="G45" s="57" t="inlineStr">
+      <c r="G46" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H45" s="58" t="inlineStr">
+      <c r="H46" s="63" t="inlineStr">
         <is>
           <t>Goiatins</t>
         </is>
       </c>
-      <c r="I45" s="58" t="inlineStr">
+      <c r="I46" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J45" s="23" t="inlineStr">
+      <c r="J46" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="57" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="62" t="inlineStr">
         <is>
           <t>7953610256</t>
         </is>
       </c>
-      <c r="B46" s="57" t="inlineStr">
+      <c r="B47" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C46" s="58" t="inlineStr">
+      <c r="C47" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00050/2026</t>
         </is>
       </c>
-      <c r="D46" s="57" t="inlineStr">
+      <c r="D47" s="62" t="inlineStr">
         <is>
           <t>Muito Alto</t>
         </is>
       </c>
-      <c r="E46" s="57" t="n">
+      <c r="E47" s="62" t="n">
         <v>111</v>
       </c>
-      <c r="G46" s="57" t="inlineStr">
+      <c r="G47" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H46" s="58" t="inlineStr">
+      <c r="H47" s="63" t="inlineStr">
         <is>
           <t>Mateiros</t>
         </is>
       </c>
-      <c r="I46" s="58" t="inlineStr">
+      <c r="I47" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J46" s="23" t="inlineStr">
+      <c r="J47" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="57" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="62" t="inlineStr">
         <is>
           <t>7926442035</t>
         </is>
       </c>
-      <c r="B47" s="57" t="inlineStr">
+      <c r="B48" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C47" s="58" t="inlineStr">
+      <c r="C48" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00051/2026</t>
         </is>
       </c>
-      <c r="D47" s="57" t="inlineStr">
+      <c r="D48" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E47" s="57" t="n">
+      <c r="E48" s="62" t="n">
         <v>111</v>
       </c>
-      <c r="G47" s="57" t="inlineStr">
+      <c r="G48" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H47" s="58" t="inlineStr">
+      <c r="H48" s="63" t="inlineStr">
         <is>
           <t>Monte Do Carmo</t>
         </is>
       </c>
-      <c r="I47" s="58" t="inlineStr">
+      <c r="I48" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J47" s="23" t="inlineStr">
+      <c r="J48" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="57" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="62" t="inlineStr">
         <is>
           <t>7925744087</t>
         </is>
       </c>
-      <c r="B48" s="57" t="inlineStr">
+      <c r="B49" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C48" s="58" t="inlineStr">
+      <c r="C49" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00059/2026</t>
         </is>
       </c>
-      <c r="D48" s="57" t="inlineStr">
+      <c r="D49" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E48" s="57" t="n">
+      <c r="E49" s="62" t="n">
         <v>99</v>
       </c>
-      <c r="G48" s="57" t="inlineStr">
+      <c r="G49" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H48" s="58" t="inlineStr">
+      <c r="H49" s="63" t="inlineStr">
         <is>
           <t>Goianorte</t>
         </is>
       </c>
-      <c r="I48" s="58" t="inlineStr">
+      <c r="I49" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J48" s="23" t="inlineStr">
+      <c r="J49" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="57" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="62" t="inlineStr">
         <is>
           <t>7925733015</t>
         </is>
       </c>
-      <c r="B49" s="57" t="inlineStr">
+      <c r="B50" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C49" s="58" t="inlineStr">
+      <c r="C50" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00058/2026</t>
         </is>
       </c>
-      <c r="D49" s="57" t="inlineStr">
+      <c r="D50" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E49" s="57" t="n">
+      <c r="E50" s="62" t="n">
         <v>99</v>
       </c>
-      <c r="G49" s="57" t="inlineStr">
+      <c r="G50" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H49" s="58" t="inlineStr">
+      <c r="H50" s="63" t="inlineStr">
         <is>
           <t>Pedro Afonso</t>
         </is>
       </c>
-      <c r="I49" s="58" t="inlineStr">
+      <c r="I50" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J49" s="23" t="inlineStr">
+      <c r="J50" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="57" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="62" t="inlineStr">
         <is>
           <t>7901110084</t>
         </is>
       </c>
-      <c r="B50" s="57" t="inlineStr">
+      <c r="B51" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C50" s="58" t="inlineStr">
+      <c r="C51" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00061/2026</t>
         </is>
       </c>
-      <c r="D50" s="57" t="inlineStr">
+      <c r="D51" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E50" s="57" t="n">
+      <c r="E51" s="62" t="n">
         <v>98</v>
       </c>
-      <c r="G50" s="57" t="inlineStr">
+      <c r="G51" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H50" s="58" t="inlineStr">
+      <c r="H51" s="63" t="inlineStr">
         <is>
           <t>Divinopolis</t>
         </is>
       </c>
-      <c r="I50" s="58" t="inlineStr">
+      <c r="I51" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J50" s="23" t="inlineStr">
+      <c r="J51" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="57" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="62" t="inlineStr">
         <is>
           <t>7944559149</t>
         </is>
       </c>
-      <c r="B51" s="57" t="inlineStr">
+      <c r="B52" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C51" s="58" t="inlineStr">
+      <c r="C52" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00063/2026</t>
         </is>
       </c>
-      <c r="D51" s="57" t="inlineStr">
+      <c r="D52" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E51" s="57" t="n">
+      <c r="E52" s="62" t="n">
         <v>98</v>
       </c>
-      <c r="G51" s="57" t="inlineStr">
+      <c r="G52" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H51" s="58" t="inlineStr">
+      <c r="H52" s="63" t="inlineStr">
         <is>
           <t>Caseara</t>
         </is>
       </c>
-      <c r="I51" s="58" t="inlineStr">
+      <c r="I52" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J51" s="23" t="inlineStr">
+      <c r="J52" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="57" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="62" t="inlineStr">
         <is>
           <t>5800291035</t>
         </is>
       </c>
-      <c r="B52" s="57" t="inlineStr">
+      <c r="B53" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C52" s="58" t="inlineStr">
+      <c r="C53" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PO 00097/2026</t>
         </is>
       </c>
-      <c r="D52" s="57" t="inlineStr">
+      <c r="D53" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E52" s="57" t="n">
+      <c r="E53" s="62" t="n">
         <v>98</v>
       </c>
-      <c r="G52" s="57" t="inlineStr">
+      <c r="G53" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H52" s="58" t="inlineStr">
+      <c r="H53" s="63" t="inlineStr">
         <is>
           <t>Monte Do Carmo</t>
         </is>
       </c>
-      <c r="I52" s="59" t="inlineStr">
+      <c r="I53" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J52" s="23" t="inlineStr">
+      <c r="J53" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="57" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="62" t="inlineStr">
         <is>
           <t>7919270014</t>
         </is>
       </c>
-      <c r="B53" s="57" t="inlineStr">
+      <c r="B54" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C53" s="58" t="inlineStr">
+      <c r="C54" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00074/2026</t>
         </is>
       </c>
-      <c r="D53" s="57" t="inlineStr">
+      <c r="D54" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E53" s="57" t="n">
+      <c r="E54" s="62" t="n">
         <v>82</v>
       </c>
-      <c r="G53" s="57" t="inlineStr">
+      <c r="G54" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H53" s="58" t="inlineStr">
+      <c r="H54" s="63" t="inlineStr">
         <is>
           <t>Pium</t>
         </is>
       </c>
-      <c r="I53" s="58" t="inlineStr">
+      <c r="I54" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J53" s="23" t="inlineStr">
+      <c r="J54" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="57" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="62" t="inlineStr">
         <is>
           <t>5801866013</t>
         </is>
       </c>
-      <c r="B54" s="57" t="inlineStr">
+      <c r="B55" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C54" s="58" t="inlineStr">
+      <c r="C55" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00077/2026</t>
         </is>
       </c>
-      <c r="D54" s="57" t="inlineStr">
+      <c r="D55" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E54" s="57" t="n">
+      <c r="E55" s="62" t="n">
         <v>79</v>
       </c>
-      <c r="G54" s="57" t="inlineStr">
+      <c r="G55" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H54" s="58" t="inlineStr">
+      <c r="H55" s="63" t="inlineStr">
         <is>
           <t>Paraiso Do Tocantins</t>
         </is>
       </c>
-      <c r="I54" s="58" t="inlineStr">
+      <c r="I55" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J54" s="23" t="inlineStr">
+      <c r="J55" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="57" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="62" t="inlineStr">
         <is>
           <t>7926089013</t>
         </is>
       </c>
-      <c r="B55" s="57" t="inlineStr">
+      <c r="B56" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C55" s="58" t="inlineStr">
+      <c r="C56" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00078/2026</t>
         </is>
       </c>
-      <c r="D55" s="57" t="inlineStr">
+      <c r="D56" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E55" s="57" t="n">
+      <c r="E56" s="62" t="n">
         <v>76</v>
       </c>
-      <c r="G55" s="57" t="inlineStr">
+      <c r="G56" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H55" s="58" t="inlineStr">
+      <c r="H56" s="63" t="inlineStr">
         <is>
           <t>Paraiso Do Tocantins</t>
         </is>
       </c>
-      <c r="I55" s="58" t="inlineStr">
+      <c r="I56" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J55" s="23" t="inlineStr">
+      <c r="J56" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="57" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="62" t="inlineStr">
         <is>
           <t>7900573047</t>
         </is>
       </c>
-      <c r="B56" s="57" t="inlineStr">
+      <c r="B57" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C56" s="58" t="inlineStr">
+      <c r="C57" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00080/2026</t>
         </is>
       </c>
-      <c r="D56" s="57" t="inlineStr">
+      <c r="D57" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E56" s="57" t="n">
+      <c r="E57" s="62" t="n">
         <v>75</v>
       </c>
-      <c r="G56" s="57" t="inlineStr">
+      <c r="G57" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H56" s="58" t="inlineStr">
+      <c r="H57" s="63" t="inlineStr">
         <is>
           <t>Figueiropolis</t>
         </is>
       </c>
-      <c r="I56" s="58" t="inlineStr">
+      <c r="I57" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J56" s="23" t="inlineStr">
+      <c r="J57" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="57" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="62" t="inlineStr">
         <is>
           <t>7927413001</t>
         </is>
       </c>
-      <c r="B57" s="57" t="inlineStr">
+      <c r="B58" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C57" s="58" t="inlineStr">
+      <c r="C58" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PO 00118/2026</t>
         </is>
       </c>
-      <c r="D57" s="57" t="inlineStr">
+      <c r="D58" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E57" s="57" t="n">
+      <c r="E58" s="62" t="n">
         <v>75</v>
       </c>
-      <c r="G57" s="57" t="inlineStr">
+      <c r="G58" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H57" s="58" t="inlineStr">
+      <c r="H58" s="63" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I57" s="59" t="inlineStr">
+      <c r="I58" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J57" s="23" t="inlineStr">
+      <c r="J58" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="57" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="62" t="inlineStr">
         <is>
           <t>7908686014</t>
         </is>
       </c>
-      <c r="B58" s="57" t="inlineStr">
+      <c r="B59" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C58" s="58" t="inlineStr">
+      <c r="C59" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00086/2026</t>
         </is>
       </c>
-      <c r="D58" s="57" t="inlineStr">
+      <c r="D59" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E58" s="57" t="n">
+      <c r="E59" s="62" t="n">
         <v>74</v>
       </c>
-      <c r="G58" s="57" t="inlineStr">
+      <c r="G59" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H58" s="58" t="inlineStr">
+      <c r="H59" s="63" t="inlineStr">
         <is>
           <t>Pium</t>
         </is>
       </c>
-      <c r="I58" s="58" t="inlineStr">
+      <c r="I59" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J58" s="23" t="inlineStr">
+      <c r="J59" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="57" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="62" t="inlineStr">
         <is>
           <t>7900117013</t>
         </is>
       </c>
-      <c r="B59" s="57" t="inlineStr">
+      <c r="B60" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C59" s="58" t="inlineStr">
+      <c r="C60" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00084/2026</t>
         </is>
       </c>
-      <c r="D59" s="57" t="inlineStr">
+      <c r="D60" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E59" s="57" t="n">
+      <c r="E60" s="62" t="n">
         <v>74</v>
       </c>
-      <c r="G59" s="57" t="inlineStr">
+      <c r="G60" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H59" s="58" t="inlineStr">
+      <c r="H60" s="63" t="inlineStr">
         <is>
           <t>Paraiso Do Tocantins</t>
         </is>
       </c>
-      <c r="I59" s="58" t="inlineStr">
+      <c r="I60" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J59" s="23" t="inlineStr">
+      <c r="J60" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="57" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="62" t="inlineStr">
         <is>
           <t>7900453110</t>
         </is>
       </c>
-      <c r="B60" s="57" t="inlineStr">
+      <c r="B61" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C60" s="58" t="inlineStr">
+      <c r="C61" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00087/2026</t>
         </is>
       </c>
-      <c r="D60" s="57" t="inlineStr">
+      <c r="D61" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E60" s="57" t="n">
+      <c r="E61" s="62" t="n">
         <v>71</v>
       </c>
-      <c r="G60" s="57" t="inlineStr">
+      <c r="G61" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H60" s="58" t="inlineStr">
+      <c r="H61" s="63" t="inlineStr">
         <is>
           <t>Santa Rita Do Tocantins</t>
         </is>
       </c>
-      <c r="I60" s="58" t="inlineStr">
+      <c r="I61" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J60" s="23" t="inlineStr">
+      <c r="J61" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="57" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="62" t="inlineStr">
         <is>
           <t>5865120195</t>
         </is>
       </c>
-      <c r="B61" s="57" t="inlineStr">
+      <c r="B62" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C61" s="58" t="inlineStr">
+      <c r="C62" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-GR 00538/2026</t>
         </is>
       </c>
-      <c r="D61" s="57" t="inlineStr">
+      <c r="D62" s="62" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E61" s="57" t="n">
+      <c r="E62" s="62" t="n">
         <v>51</v>
       </c>
-      <c r="G61" s="57" t="inlineStr">
+      <c r="G62" s="62" t="inlineStr">
         <is>
           <t>COCM-N</t>
         </is>
       </c>
-      <c r="H61" s="58" t="inlineStr">
+      <c r="H62" s="63" t="inlineStr">
         <is>
           <t>Centenario</t>
         </is>
       </c>
-      <c r="I61" s="59" t="inlineStr">
+      <c r="I62" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J61" s="23" t="inlineStr">
+      <c r="J62" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="57" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="62" t="inlineStr">
         <is>
           <t>5836786094</t>
         </is>
       </c>
-      <c r="B62" s="57" t="inlineStr">
+      <c r="B63" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C62" s="58" t="inlineStr">
+      <c r="C63" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00095/2026</t>
         </is>
       </c>
-      <c r="D62" s="57" t="inlineStr">
+      <c r="D63" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E62" s="57" t="n">
+      <c r="E63" s="62" t="n">
         <v>50</v>
       </c>
-      <c r="G62" s="57" t="inlineStr">
+      <c r="G63" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H62" s="58" t="inlineStr">
+      <c r="H63" s="63" t="inlineStr">
         <is>
           <t>Peixe</t>
         </is>
       </c>
-      <c r="I62" s="58" t="inlineStr">
+      <c r="I63" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J62" s="23" t="inlineStr">
+      <c r="J63" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="57" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="62" t="inlineStr">
         <is>
           <t>7900594026</t>
         </is>
       </c>
-      <c r="B63" s="57" t="inlineStr">
+      <c r="B64" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C63" s="58" t="inlineStr">
+      <c r="C64" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00113/2026</t>
         </is>
       </c>
-      <c r="D63" s="57" t="inlineStr">
+      <c r="D64" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E63" s="57" t="n">
+      <c r="E64" s="62" t="n">
         <v>27</v>
       </c>
-      <c r="G63" s="57" t="inlineStr">
+      <c r="G64" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H63" s="58" t="inlineStr">
+      <c r="H64" s="63" t="inlineStr">
         <is>
           <t>Ponte Alta Tocantins</t>
         </is>
       </c>
-      <c r="I63" s="58" t="inlineStr">
+      <c r="I64" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J63" s="23" t="inlineStr">
+      <c r="J64" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="57" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="62" t="inlineStr">
         <is>
           <t>7913662076</t>
         </is>
       </c>
-      <c r="B64" s="57" t="inlineStr">
+      <c r="B65" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C64" s="58" t="inlineStr">
+      <c r="C65" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00114/2026</t>
         </is>
       </c>
-      <c r="D64" s="57" t="inlineStr">
+      <c r="D65" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E64" s="57" t="n">
+      <c r="E65" s="62" t="n">
         <v>27</v>
       </c>
-      <c r="G64" s="57" t="inlineStr">
+      <c r="G65" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H64" s="58" t="inlineStr">
+      <c r="H65" s="63" t="inlineStr">
         <is>
           <t>Duere</t>
         </is>
       </c>
-      <c r="I64" s="58" t="inlineStr">
+      <c r="I65" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J64" s="23" t="inlineStr">
+      <c r="J65" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="57" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="62" t="inlineStr">
         <is>
           <t>5800859011</t>
         </is>
       </c>
-      <c r="B65" s="57" t="inlineStr">
+      <c r="B66" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C65" s="58" t="inlineStr">
+      <c r="C66" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00115/2026</t>
         </is>
       </c>
-      <c r="D65" s="57" t="inlineStr">
+      <c r="D66" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E65" s="57" t="n">
+      <c r="E66" s="62" t="n">
         <v>25</v>
       </c>
-      <c r="G65" s="57" t="inlineStr">
+      <c r="G66" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H65" s="58" t="inlineStr">
+      <c r="H66" s="63" t="inlineStr">
         <is>
           <t>Tupirama</t>
         </is>
       </c>
-      <c r="I65" s="58" t="inlineStr">
+      <c r="I66" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J65" s="23" t="inlineStr">
+      <c r="J66" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="57" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="62" t="inlineStr">
         <is>
           <t>5800090147</t>
         </is>
       </c>
-      <c r="B66" s="57" t="inlineStr">
+      <c r="B67" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C66" s="58" t="inlineStr">
+      <c r="C67" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00117/2026</t>
         </is>
       </c>
-      <c r="D66" s="57" t="inlineStr">
+      <c r="D67" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E66" s="57" t="n">
+      <c r="E67" s="62" t="n">
         <v>22</v>
       </c>
-      <c r="G66" s="57" t="inlineStr">
+      <c r="G67" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H66" s="58" t="inlineStr">
+      <c r="H67" s="63" t="inlineStr">
         <is>
           <t>Taipas Do Tocantins</t>
         </is>
       </c>
-      <c r="I66" s="58" t="inlineStr">
+      <c r="I67" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J66" s="23" t="inlineStr">
+      <c r="J67" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="57" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="62" t="inlineStr">
         <is>
           <t>5856156091</t>
         </is>
       </c>
-      <c r="B67" s="57" t="inlineStr">
+      <c r="B68" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C67" s="58" t="inlineStr">
+      <c r="C68" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-DP 00403/2026</t>
         </is>
       </c>
-      <c r="D67" s="57" t="inlineStr">
+      <c r="D68" s="62" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E67" s="57" t="n">
+      <c r="E68" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="G67" s="57" t="inlineStr">
+      <c r="G68" s="62" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H67" s="58" t="inlineStr">
+      <c r="H68" s="63" t="inlineStr">
         <is>
           <t>Almas</t>
         </is>
       </c>
-      <c r="I67" s="59" t="inlineStr">
+      <c r="I68" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J67" s="23" t="inlineStr">
+      <c r="J68" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="57" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="62" t="inlineStr">
         <is>
           <t>5827102054</t>
         </is>
       </c>
-      <c r="B68" s="57" t="inlineStr">
+      <c r="B69" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C68" s="58" t="inlineStr">
+      <c r="C69" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PS 00289/2026</t>
         </is>
       </c>
-      <c r="D68" s="57" t="inlineStr">
+      <c r="D69" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E68" s="57" t="n">
+      <c r="E69" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="G68" s="57" t="inlineStr">
+      <c r="G69" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H68" s="58" t="inlineStr">
+      <c r="H69" s="63" t="inlineStr">
         <is>
           <t>Pugmil</t>
         </is>
       </c>
-      <c r="I68" s="58" t="inlineStr">
+      <c r="I69" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J68" s="23" t="inlineStr">
+      <c r="J69" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="57" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="62" t="inlineStr">
         <is>
           <t>5846328094</t>
         </is>
       </c>
-      <c r="B69" s="57" t="inlineStr">
+      <c r="B70" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C69" s="58" t="inlineStr">
+      <c r="C70" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-GU 00687/2026</t>
         </is>
       </c>
-      <c r="D69" s="57" t="inlineStr">
+      <c r="D70" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E69" s="57" t="n">
+      <c r="E70" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="G69" s="57" t="inlineStr">
+      <c r="G70" s="62" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H69" s="58" t="inlineStr">
+      <c r="H70" s="63" t="inlineStr">
         <is>
           <t>Peixe</t>
         </is>
       </c>
-      <c r="I69" s="59" t="inlineStr">
+      <c r="I70" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J69" s="23" t="inlineStr">
+      <c r="J70" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="57" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="62" t="inlineStr">
         <is>
           <t>7942572059</t>
         </is>
       </c>
-      <c r="B70" s="57" t="inlineStr">
+      <c r="B71" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C70" s="58" t="inlineStr">
+      <c r="C71" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00427/2026</t>
         </is>
       </c>
-      <c r="D70" s="57" t="inlineStr">
+      <c r="D71" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E70" s="57" t="n">
+      <c r="E71" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="G70" s="57" t="inlineStr">
+      <c r="G71" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H70" s="58" t="inlineStr">
+      <c r="H71" s="63" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I70" s="59" t="inlineStr">
+      <c r="I71" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J70" s="23" t="inlineStr">
+      <c r="J71" s="23" t="inlineStr">
         <is>
           <t>EXECUTADO</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="57" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="62" t="inlineStr">
         <is>
           <t>7929376022</t>
         </is>
       </c>
-      <c r="B71" s="57" t="inlineStr">
+      <c r="B72" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C71" s="58" t="inlineStr">
+      <c r="C72" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00120/2026</t>
         </is>
       </c>
-      <c r="D71" s="57" t="inlineStr">
+      <c r="D72" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E71" s="57" t="n">
+      <c r="E72" s="62" t="n">
         <v>7</v>
       </c>
-      <c r="G71" s="57" t="inlineStr">
+      <c r="G72" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H71" s="58" t="inlineStr">
+      <c r="H72" s="63" t="inlineStr">
         <is>
           <t>Babaculandia</t>
         </is>
       </c>
-      <c r="I71" s="58" t="inlineStr">
+      <c r="I72" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J71" s="23" t="inlineStr">
+      <c r="J72" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="57" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="62" t="inlineStr">
         <is>
           <t>5800438116</t>
         </is>
       </c>
-      <c r="B72" s="57" t="inlineStr">
+      <c r="B73" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C72" s="58" t="inlineStr">
+      <c r="C73" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-DP 00404/2026</t>
         </is>
       </c>
-      <c r="D72" s="57" t="inlineStr">
+      <c r="D73" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E72" s="57" t="n">
+      <c r="E73" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G72" s="57" t="inlineStr">
+      <c r="G73" s="62" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H72" s="58" t="inlineStr">
+      <c r="H73" s="63" t="inlineStr">
         <is>
           <t>Chapada Da Natividade</t>
         </is>
       </c>
-      <c r="I72" s="58" t="inlineStr">
+      <c r="I73" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J72" s="23" t="inlineStr">
+      <c r="J73" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="57" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="62" t="inlineStr">
         <is>
           <t>5803327001</t>
         </is>
       </c>
-      <c r="B73" s="57" t="inlineStr">
+      <c r="B74" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C73" s="58" t="inlineStr">
+      <c r="C74" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00434/2026</t>
         </is>
       </c>
-      <c r="D73" s="57" t="inlineStr">
+      <c r="D74" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E73" s="57" t="n">
+      <c r="E74" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G73" s="57" t="inlineStr">
+      <c r="G74" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H73" s="58" t="inlineStr">
+      <c r="H74" s="63" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I73" s="59" t="inlineStr">
+      <c r="I74" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J73" s="23" t="inlineStr">
+      <c r="J74" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="57" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="62" t="inlineStr">
         <is>
           <t>7933766059</t>
         </is>
       </c>
-      <c r="B74" s="57" t="inlineStr">
+      <c r="B75" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C74" s="58" t="inlineStr">
+      <c r="C75" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00431/2026</t>
         </is>
       </c>
-      <c r="D74" s="57" t="inlineStr">
+      <c r="D75" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E74" s="57" t="n">
+      <c r="E75" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G74" s="57" t="inlineStr">
+      <c r="G75" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H74" s="58" t="inlineStr">
+      <c r="H75" s="63" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I74" s="58" t="inlineStr">
+      <c r="I75" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J74" s="23" t="inlineStr">
+      <c r="J75" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="57" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="62" t="inlineStr">
         <is>
           <t>7931610122</t>
         </is>
       </c>
-      <c r="B75" s="57" t="inlineStr">
+      <c r="B76" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C75" s="58" t="inlineStr">
+      <c r="C76" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00433/2026</t>
         </is>
       </c>
-      <c r="D75" s="57" t="inlineStr">
+      <c r="D76" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E75" s="57" t="n">
+      <c r="E76" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G75" s="57" t="inlineStr">
+      <c r="G76" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H75" s="58" t="inlineStr">
+      <c r="H76" s="63" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I75" s="58" t="inlineStr">
+      <c r="I76" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J75" s="23" t="inlineStr">
+      <c r="J76" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="57" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="62" t="inlineStr">
         <is>
           <t>7927169001</t>
         </is>
       </c>
-      <c r="B76" s="57" t="inlineStr">
+      <c r="B77" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C76" s="58" t="inlineStr">
+      <c r="C77" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00432/2026</t>
         </is>
       </c>
-      <c r="D76" s="57" t="inlineStr">
+      <c r="D77" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E76" s="57" t="n">
+      <c r="E77" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G76" s="57" t="inlineStr">
+      <c r="G77" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H76" s="58" t="inlineStr">
+      <c r="H77" s="63" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I76" s="58" t="inlineStr">
+      <c r="I77" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J76" s="23" t="inlineStr">
+      <c r="J77" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="57" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="62" t="inlineStr">
         <is>
           <t>7933726256</t>
         </is>
       </c>
-      <c r="B77" s="57" t="inlineStr">
+      <c r="B78" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C77" s="58" t="inlineStr">
+      <c r="C78" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-PO 00181/2026</t>
         </is>
       </c>
-      <c r="D77" s="57" t="inlineStr">
+      <c r="D78" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E77" s="57" t="n">
+      <c r="E78" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G77" s="57" t="inlineStr">
+      <c r="G78" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H77" s="58" t="inlineStr">
+      <c r="H78" s="63" t="inlineStr">
         <is>
           <t>Mateiros</t>
         </is>
       </c>
-      <c r="I77" s="58" t="inlineStr">
+      <c r="I78" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J77" s="23" t="inlineStr">
+      <c r="J78" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="57" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="62" t="inlineStr">
         <is>
           <t>7911120026</t>
         </is>
       </c>
-      <c r="B78" s="57" t="inlineStr">
+      <c r="B79" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C78" s="58" t="inlineStr">
+      <c r="C79" s="63" t="inlineStr">
         <is>
           <t>DG-RD-PO 00444/2026</t>
         </is>
       </c>
-      <c r="D78" s="57" t="inlineStr">
+      <c r="D79" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E78" s="57" t="n">
+      <c r="E79" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="G78" s="57" t="inlineStr">
+      <c r="G79" s="62" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H78" s="58" t="inlineStr">
+      <c r="H79" s="63" t="inlineStr">
         <is>
           <t>Ponte Alta Tocantins</t>
         </is>
       </c>
-      <c r="I78" s="59" t="inlineStr">
+      <c r="I79" s="64" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
       </c>
-      <c r="J78" s="23" t="inlineStr">
+      <c r="J79" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="57" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="62" t="inlineStr">
         <is>
           <t>7908705049</t>
         </is>
       </c>
-      <c r="B79" s="57" t="inlineStr">
+      <c r="B80" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C79" s="58" t="inlineStr">
+      <c r="C80" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-DP 00409/2026</t>
         </is>
       </c>
-      <c r="D79" s="57" t="inlineStr">
+      <c r="D80" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E79" s="57" t="n">
+      <c r="E80" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="G79" s="57" t="inlineStr">
+      <c r="G80" s="62" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H79" s="58" t="inlineStr">
+      <c r="H80" s="63" t="inlineStr">
         <is>
           <t>Aurora Do Tocantins</t>
         </is>
       </c>
-      <c r="I79" s="58" t="inlineStr">
+      <c r="I80" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J79" s="23" t="inlineStr">
+      <c r="J80" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="57" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="62" t="inlineStr">
         <is>
           <t>7900230155</t>
         </is>
       </c>
-      <c r="B80" s="57" t="inlineStr">
+      <c r="B81" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C80" s="58" t="inlineStr">
+      <c r="C81" s="63" t="inlineStr">
         <is>
           <t>ETO-RD-GR 00685/2026</t>
         </is>
       </c>
-      <c r="D80" s="57" t="inlineStr">
+      <c r="D81" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E80" s="57" t="n">
+      <c r="E81" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G80" s="57" t="inlineStr">
+      <c r="G81" s="62" t="inlineStr">
         <is>
           <t>COCM-N</t>
         </is>
       </c>
-      <c r="H80" s="58" t="inlineStr">
+      <c r="H81" s="63" t="inlineStr">
         <is>
           <t>Palmeirante</t>
         </is>
       </c>
-      <c r="I80" s="58" t="inlineStr">
+      <c r="I81" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J80" s="23" t="inlineStr">
+      <c r="J81" s="23" t="inlineStr">
         <is>
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="57" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="62" t="inlineStr">
         <is>
           <t>7928564039</t>
         </is>
       </c>
-      <c r="B81" s="57" t="inlineStr">
+      <c r="B82" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C81" s="58" t="inlineStr">
+      <c r="C82" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00123/2026</t>
         </is>
       </c>
-      <c r="D81" s="57" t="inlineStr">
+      <c r="D82" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E81" s="57" t="n">
+      <c r="E82" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G81" s="57" t="inlineStr">
+      <c r="G82" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H81" s="58" t="inlineStr">
+      <c r="H82" s="63" t="inlineStr">
         <is>
           <t>Araguatins</t>
         </is>
       </c>
-      <c r="I81" s="58" t="inlineStr">
+      <c r="I82" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J81" s="23" t="inlineStr">
+      <c r="J82" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="57" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="62" t="inlineStr">
         <is>
           <t>7928241200</t>
         </is>
       </c>
-      <c r="B82" s="57" t="inlineStr">
+      <c r="B83" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C82" s="58" t="inlineStr">
+      <c r="C83" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00128/2026</t>
         </is>
       </c>
-      <c r="D82" s="57" t="inlineStr">
+      <c r="D83" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E82" s="57" t="n">
+      <c r="E83" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G82" s="57" t="inlineStr">
+      <c r="G83" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H82" s="58" t="inlineStr">
+      <c r="H83" s="63" t="inlineStr">
         <is>
           <t>Sao Salvador Do Tocantins</t>
         </is>
       </c>
-      <c r="I82" s="58" t="inlineStr">
+      <c r="I83" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J82" s="23" t="inlineStr">
+      <c r="J83" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="57" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="62" t="inlineStr">
         <is>
           <t>5856070091</t>
         </is>
       </c>
-      <c r="B83" s="57" t="inlineStr">
+      <c r="B84" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C83" s="58" t="inlineStr">
+      <c r="C84" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00130/2026</t>
         </is>
       </c>
-      <c r="D83" s="57" t="inlineStr">
+      <c r="D84" s="62" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E83" s="57" t="n">
+      <c r="E84" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G83" s="57" t="inlineStr">
+      <c r="G84" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H83" s="58" t="inlineStr">
+      <c r="H84" s="63" t="inlineStr">
         <is>
           <t>Almas</t>
         </is>
       </c>
-      <c r="I83" s="58" t="inlineStr">
+      <c r="I84" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J83" s="23" t="inlineStr">
+      <c r="J84" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="57" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="62" t="inlineStr">
         <is>
           <t>5850308009</t>
         </is>
       </c>
-      <c r="B84" s="57" t="inlineStr">
+      <c r="B85" s="62" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C84" s="58" t="inlineStr">
+      <c r="C85" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00127/2026</t>
         </is>
       </c>
-      <c r="D84" s="57" t="inlineStr">
+      <c r="D85" s="62" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E84" s="57" t="n">
+      <c r="E85" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G84" s="57" t="inlineStr">
+      <c r="G85" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H84" s="58" t="inlineStr">
+      <c r="H85" s="63" t="inlineStr">
         <is>
           <t>Guarai</t>
         </is>
       </c>
-      <c r="I84" s="58" t="inlineStr">
+      <c r="I85" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J84" s="23" t="inlineStr">
+      <c r="J85" s="23" t="inlineStr">
         <is>
           <t>CONCLUÍDA MAS AINDA NO POSTO (VERIFICAR)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="57" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="62" t="inlineStr">
         <is>
           <t>7937102148</t>
         </is>
       </c>
-      <c r="B85" s="57" t="inlineStr">
+      <c r="B86" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C85" s="58" t="inlineStr">
+      <c r="C86" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00129/2026</t>
         </is>
       </c>
-      <c r="D85" s="57" t="inlineStr">
+      <c r="D86" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E85" s="57" t="n">
+      <c r="E86" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G85" s="57" t="inlineStr">
+      <c r="G86" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H85" s="58" t="inlineStr">
+      <c r="H86" s="63" t="inlineStr">
         <is>
           <t>Sao Valerio Da Natividade</t>
         </is>
       </c>
-      <c r="I85" s="58" t="inlineStr">
+      <c r="I86" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J85" s="23" t="inlineStr">
+      <c r="J86" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="57" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="62" t="inlineStr">
         <is>
           <t>7923673004</t>
         </is>
       </c>
-      <c r="B86" s="57" t="inlineStr">
+      <c r="B87" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C86" s="58" t="inlineStr">
+      <c r="C87" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00124/2026</t>
         </is>
       </c>
-      <c r="D86" s="57" t="inlineStr">
+      <c r="D87" s="62" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E86" s="57" t="n">
+      <c r="E87" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G86" s="57" t="inlineStr">
+      <c r="G87" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H86" s="58" t="inlineStr">
+      <c r="H87" s="63" t="inlineStr">
         <is>
           <t>Araguaina</t>
         </is>
       </c>
-      <c r="I86" s="58" t="inlineStr">
+      <c r="I87" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J86" s="23" t="inlineStr">
+      <c r="J87" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="57" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="62" t="inlineStr">
         <is>
           <t>7900525015</t>
         </is>
       </c>
-      <c r="B87" s="57" t="inlineStr">
+      <c r="B88" s="62" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C87" s="58" t="inlineStr">
+      <c r="C88" s="63" t="inlineStr">
         <is>
           <t>ETO-COEP 00125/2026</t>
         </is>
       </c>
-      <c r="D87" s="57" t="inlineStr">
+      <c r="D88" s="62" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E87" s="57" t="n">
+      <c r="E88" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G87" s="57" t="inlineStr">
+      <c r="G88" s="62" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H87" s="58" t="inlineStr">
+      <c r="H88" s="63" t="inlineStr">
         <is>
           <t>Pedro Afonso</t>
         </is>
       </c>
-      <c r="I87" s="58" t="inlineStr">
+      <c r="I88" s="63" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
       </c>
-      <c r="J87" s="23" t="inlineStr">
+      <c r="J88" s="23" t="inlineStr">
         <is>
           <t>No posto do COEP (pendente)</t>
         </is>

</xml_diff>

<commit_message>
Registra confirmação do SGM no caso do trafo de Pium (7931219078)
Cadeia ETO-TELE 00694/2025 > ETO-COEP 00163/2025 (encerrada: não é
responsabilidade da área) > ETO-RD-PO 00180/2026 (COCM) e ETO-TELE 00975/2026
anotada na observação — confirma o tratamento sem compra COEP

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBtNB8AfUGxQoc5b1rirVp
</commit_message>
<xml_diff>
--- a/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
+++ b/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -315,15 +315,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2933,40 +2924,40 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="62" t="inlineStr">
+      <c r="A24" s="57" t="inlineStr">
         <is>
           <t>7923927122</t>
         </is>
       </c>
-      <c r="B24" s="62" t="inlineStr">
+      <c r="B24" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C24" s="63" t="inlineStr">
+      <c r="C24" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00079/2025</t>
         </is>
       </c>
-      <c r="D24" s="62" t="inlineStr">
+      <c r="D24" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E24" s="62" t="n">
+      <c r="E24" s="57" t="n">
         <v>434</v>
       </c>
-      <c r="G24" s="62" t="inlineStr">
+      <c r="G24" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H24" s="63" t="inlineStr">
+      <c r="H24" s="58" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I24" s="63" t="inlineStr">
+      <c r="I24" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -2978,40 +2969,40 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="62" t="inlineStr">
+      <c r="A25" s="57" t="inlineStr">
         <is>
           <t>7900532053</t>
         </is>
       </c>
-      <c r="B25" s="62" t="inlineStr">
+      <c r="B25" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C25" s="63" t="inlineStr">
+      <c r="C25" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00102/2025</t>
         </is>
       </c>
-      <c r="D25" s="62" t="inlineStr">
+      <c r="D25" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E25" s="62" t="n">
+      <c r="E25" s="57" t="n">
         <v>407</v>
       </c>
-      <c r="G25" s="62" t="inlineStr">
+      <c r="G25" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H25" s="63" t="inlineStr">
+      <c r="H25" s="58" t="inlineStr">
         <is>
           <t>Piraque</t>
         </is>
       </c>
-      <c r="I25" s="63" t="inlineStr">
+      <c r="I25" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3023,40 +3014,40 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="62" t="inlineStr">
+      <c r="A26" s="57" t="inlineStr">
         <is>
           <t>7920024127</t>
         </is>
       </c>
-      <c r="B26" s="62" t="inlineStr">
+      <c r="B26" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C26" s="63" t="inlineStr">
+      <c r="C26" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00120/2025</t>
         </is>
       </c>
-      <c r="D26" s="62" t="inlineStr">
+      <c r="D26" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E26" s="62" t="n">
+      <c r="E26" s="57" t="n">
         <v>371</v>
       </c>
-      <c r="G26" s="62" t="inlineStr">
+      <c r="G26" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H26" s="63" t="inlineStr">
+      <c r="H26" s="58" t="inlineStr">
         <is>
           <t>Palmeiras Do Tocantins</t>
         </is>
       </c>
-      <c r="I26" s="63" t="inlineStr">
+      <c r="I26" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3068,40 +3059,40 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="62" t="inlineStr">
+      <c r="A27" s="57" t="inlineStr">
         <is>
           <t>5858783119</t>
         </is>
       </c>
-      <c r="B27" s="62" t="inlineStr">
+      <c r="B27" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C27" s="63" t="inlineStr">
+      <c r="C27" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00123/2025</t>
         </is>
       </c>
-      <c r="D27" s="62" t="inlineStr">
+      <c r="D27" s="57" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E27" s="62" t="n">
+      <c r="E27" s="57" t="n">
         <v>369</v>
       </c>
-      <c r="G27" s="62" t="inlineStr">
+      <c r="G27" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H27" s="63" t="inlineStr">
+      <c r="H27" s="58" t="inlineStr">
         <is>
           <t>Sao Bento Do Tocantins</t>
         </is>
       </c>
-      <c r="I27" s="63" t="inlineStr">
+      <c r="I27" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3113,40 +3104,40 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="62" t="inlineStr">
+      <c r="A28" s="57" t="inlineStr">
         <is>
           <t>7927446001</t>
         </is>
       </c>
-      <c r="B28" s="62" t="inlineStr">
+      <c r="B28" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C28" s="63" t="inlineStr">
+      <c r="C28" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00143/2025</t>
         </is>
       </c>
-      <c r="D28" s="62" t="inlineStr">
+      <c r="D28" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E28" s="62" t="n">
+      <c r="E28" s="57" t="n">
         <v>364</v>
       </c>
-      <c r="G28" s="62" t="inlineStr">
+      <c r="G28" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H28" s="63" t="inlineStr">
+      <c r="H28" s="58" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I28" s="63" t="inlineStr">
+      <c r="I28" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3158,40 +3149,40 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="62" t="inlineStr">
+      <c r="A29" s="57" t="inlineStr">
         <is>
           <t>7957126085</t>
         </is>
       </c>
-      <c r="B29" s="62" t="inlineStr">
+      <c r="B29" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C29" s="63" t="inlineStr">
+      <c r="C29" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00156/2025</t>
         </is>
       </c>
-      <c r="D29" s="62" t="inlineStr">
+      <c r="D29" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E29" s="62" t="n">
+      <c r="E29" s="57" t="n">
         <v>350</v>
       </c>
-      <c r="G29" s="62" t="inlineStr">
+      <c r="G29" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H29" s="63" t="inlineStr">
+      <c r="H29" s="58" t="inlineStr">
         <is>
           <t>Monte Santo Do Tocantins</t>
         </is>
       </c>
-      <c r="I29" s="63" t="inlineStr">
+      <c r="I29" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3203,40 +3194,40 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="62" t="inlineStr">
+      <c r="A30" s="57" t="inlineStr">
         <is>
           <t>7942485096</t>
         </is>
       </c>
-      <c r="B30" s="62" t="inlineStr">
+      <c r="B30" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C30" s="63" t="inlineStr">
+      <c r="C30" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00158/2025</t>
         </is>
       </c>
-      <c r="D30" s="62" t="inlineStr">
+      <c r="D30" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E30" s="62" t="n">
+      <c r="E30" s="57" t="n">
         <v>349</v>
       </c>
-      <c r="G30" s="62" t="inlineStr">
+      <c r="G30" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H30" s="63" t="inlineStr">
+      <c r="H30" s="58" t="inlineStr">
         <is>
           <t>Pindorama Do Tocantins</t>
         </is>
       </c>
-      <c r="I30" s="63" t="inlineStr">
+      <c r="I30" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3248,40 +3239,40 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="62" t="inlineStr">
+      <c r="A31" s="57" t="inlineStr">
         <is>
           <t>5854566043</t>
         </is>
       </c>
-      <c r="B31" s="62" t="inlineStr">
+      <c r="B31" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C31" s="63" t="inlineStr">
+      <c r="C31" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00160/2025</t>
         </is>
       </c>
-      <c r="D31" s="62" t="inlineStr">
+      <c r="D31" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E31" s="62" t="n">
+      <c r="E31" s="57" t="n">
         <v>347</v>
       </c>
-      <c r="G31" s="62" t="inlineStr">
+      <c r="G31" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H31" s="63" t="inlineStr">
+      <c r="H31" s="58" t="inlineStr">
         <is>
           <t>Silvanopolis</t>
         </is>
       </c>
-      <c r="I31" s="63" t="inlineStr">
+      <c r="I31" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3293,40 +3284,40 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="62" t="inlineStr">
+      <c r="A32" s="57" t="inlineStr">
         <is>
           <t>5844630060</t>
         </is>
       </c>
-      <c r="B32" s="62" t="inlineStr">
+      <c r="B32" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C32" s="63" t="inlineStr">
+      <c r="C32" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00167/2025</t>
         </is>
       </c>
-      <c r="D32" s="62" t="inlineStr">
+      <c r="D32" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E32" s="62" t="n">
+      <c r="E32" s="57" t="n">
         <v>333</v>
       </c>
-      <c r="G32" s="62" t="inlineStr">
+      <c r="G32" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H32" s="63" t="inlineStr">
+      <c r="H32" s="58" t="inlineStr">
         <is>
           <t>Nova Olinda</t>
         </is>
       </c>
-      <c r="I32" s="63" t="inlineStr">
+      <c r="I32" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3338,40 +3329,40 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="62" t="inlineStr">
+      <c r="A33" s="57" t="inlineStr">
         <is>
           <t>7900535058</t>
         </is>
       </c>
-      <c r="B33" s="62" t="inlineStr">
+      <c r="B33" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C33" s="63" t="inlineStr">
+      <c r="C33" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00173/2025</t>
         </is>
       </c>
-      <c r="D33" s="62" t="inlineStr">
+      <c r="D33" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E33" s="62" t="n">
+      <c r="E33" s="57" t="n">
         <v>317</v>
       </c>
-      <c r="G33" s="62" t="inlineStr">
+      <c r="G33" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H33" s="63" t="inlineStr">
+      <c r="H33" s="58" t="inlineStr">
         <is>
           <t>Santa Fe Do Araguaia</t>
         </is>
       </c>
-      <c r="I33" s="63" t="inlineStr">
+      <c r="I33" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3383,40 +3374,40 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="62" t="inlineStr">
+      <c r="A34" s="57" t="inlineStr">
         <is>
           <t>7903112004</t>
         </is>
       </c>
-      <c r="B34" s="62" t="inlineStr">
+      <c r="B34" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C34" s="63" t="inlineStr">
+      <c r="C34" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00184/2025</t>
         </is>
       </c>
-      <c r="D34" s="62" t="inlineStr">
+      <c r="D34" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E34" s="62" t="n">
+      <c r="E34" s="57" t="n">
         <v>307</v>
       </c>
-      <c r="G34" s="62" t="inlineStr">
+      <c r="G34" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H34" s="63" t="inlineStr">
+      <c r="H34" s="58" t="inlineStr">
         <is>
           <t>Araguaina</t>
         </is>
       </c>
-      <c r="I34" s="63" t="inlineStr">
+      <c r="I34" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3428,40 +3419,40 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="62" t="inlineStr">
+      <c r="A35" s="57" t="inlineStr">
         <is>
           <t>5800371025</t>
         </is>
       </c>
-      <c r="B35" s="62" t="inlineStr">
+      <c r="B35" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C35" s="63" t="inlineStr">
+      <c r="C35" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00187/2025</t>
         </is>
       </c>
-      <c r="D35" s="62" t="inlineStr">
+      <c r="D35" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E35" s="62" t="n">
+      <c r="E35" s="57" t="n">
         <v>305</v>
       </c>
-      <c r="G35" s="62" t="inlineStr">
+      <c r="G35" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H35" s="63" t="inlineStr">
+      <c r="H35" s="58" t="inlineStr">
         <is>
           <t>Arapoema</t>
         </is>
       </c>
-      <c r="I35" s="63" t="inlineStr">
+      <c r="I35" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3473,40 +3464,40 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="62" t="inlineStr">
+      <c r="A36" s="57" t="inlineStr">
         <is>
           <t>5855411017</t>
         </is>
       </c>
-      <c r="B36" s="62" t="inlineStr">
+      <c r="B36" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C36" s="63" t="inlineStr">
+      <c r="C36" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00199/2025</t>
         </is>
       </c>
-      <c r="D36" s="62" t="inlineStr">
+      <c r="D36" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E36" s="62" t="n">
+      <c r="E36" s="57" t="n">
         <v>280</v>
       </c>
-      <c r="G36" s="62" t="inlineStr">
+      <c r="G36" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H36" s="63" t="inlineStr">
+      <c r="H36" s="58" t="inlineStr">
         <is>
           <t>Barrolandia</t>
         </is>
       </c>
-      <c r="I36" s="63" t="inlineStr">
+      <c r="I36" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3518,40 +3509,40 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="62" t="inlineStr">
+      <c r="A37" s="57" t="inlineStr">
         <is>
           <t>5853360007</t>
         </is>
       </c>
-      <c r="B37" s="62" t="inlineStr">
+      <c r="B37" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C37" s="63" t="inlineStr">
+      <c r="C37" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PS 00323/2025</t>
         </is>
       </c>
-      <c r="D37" s="62" t="inlineStr">
+      <c r="D37" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E37" s="62" t="n">
+      <c r="E37" s="57" t="n">
         <v>264</v>
       </c>
-      <c r="G37" s="62" t="inlineStr">
+      <c r="G37" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H37" s="63" t="inlineStr">
+      <c r="H37" s="58" t="inlineStr">
         <is>
           <t>Miracema Do Tocantins</t>
         </is>
       </c>
-      <c r="I37" s="64" t="inlineStr">
+      <c r="I37" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -3563,40 +3554,40 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="62" t="inlineStr">
+      <c r="A38" s="57" t="inlineStr">
         <is>
           <t>5800961074</t>
         </is>
       </c>
-      <c r="B38" s="62" t="inlineStr">
+      <c r="B38" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C38" s="63" t="inlineStr">
+      <c r="C38" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00221/2025</t>
         </is>
       </c>
-      <c r="D38" s="62" t="inlineStr">
+      <c r="D38" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E38" s="62" t="n">
+      <c r="E38" s="57" t="n">
         <v>214</v>
       </c>
-      <c r="G38" s="62" t="inlineStr">
+      <c r="G38" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H38" s="63" t="inlineStr">
+      <c r="H38" s="58" t="inlineStr">
         <is>
           <t>Dianopolis</t>
         </is>
       </c>
-      <c r="I38" s="63" t="inlineStr">
+      <c r="I38" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3608,40 +3599,40 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="62" t="inlineStr">
+      <c r="A39" s="57" t="inlineStr">
         <is>
           <t>7925087021</t>
         </is>
       </c>
-      <c r="B39" s="62" t="inlineStr">
+      <c r="B39" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C39" s="63" t="inlineStr">
+      <c r="C39" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00222/2025</t>
         </is>
       </c>
-      <c r="D39" s="62" t="inlineStr">
+      <c r="D39" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E39" s="62" t="n">
+      <c r="E39" s="57" t="n">
         <v>211</v>
       </c>
-      <c r="G39" s="62" t="inlineStr">
+      <c r="G39" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H39" s="63" t="inlineStr">
+      <c r="H39" s="58" t="inlineStr">
         <is>
           <t>Parana</t>
         </is>
       </c>
-      <c r="I39" s="63" t="inlineStr">
+      <c r="I39" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3653,40 +3644,40 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="62" t="inlineStr">
+      <c r="A40" s="57" t="inlineStr">
         <is>
           <t>5862236091</t>
         </is>
       </c>
-      <c r="B40" s="62" t="inlineStr">
+      <c r="B40" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C40" s="63" t="inlineStr">
+      <c r="C40" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00223/2025</t>
         </is>
       </c>
-      <c r="D40" s="62" t="inlineStr">
+      <c r="D40" s="57" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E40" s="62" t="n">
+      <c r="E40" s="57" t="n">
         <v>211</v>
       </c>
-      <c r="G40" s="62" t="inlineStr">
+      <c r="G40" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H40" s="63" t="inlineStr">
+      <c r="H40" s="58" t="inlineStr">
         <is>
           <t>Almas</t>
         </is>
       </c>
-      <c r="I40" s="63" t="inlineStr">
+      <c r="I40" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3698,40 +3689,40 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="62" t="inlineStr">
+      <c r="A41" s="57" t="inlineStr">
         <is>
           <t>7933585074</t>
         </is>
       </c>
-      <c r="B41" s="62" t="inlineStr">
+      <c r="B41" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C41" s="63" t="inlineStr">
+      <c r="C41" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00024/2026</t>
         </is>
       </c>
-      <c r="D41" s="62" t="inlineStr">
+      <c r="D41" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E41" s="62" t="n">
+      <c r="E41" s="57" t="n">
         <v>161</v>
       </c>
-      <c r="G41" s="62" t="inlineStr">
+      <c r="G41" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H41" s="63" t="inlineStr">
+      <c r="H41" s="58" t="inlineStr">
         <is>
           <t>Dianopolis</t>
         </is>
       </c>
-      <c r="I41" s="63" t="inlineStr">
+      <c r="I41" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3743,40 +3734,40 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="62" t="inlineStr">
+      <c r="A42" s="57" t="inlineStr">
         <is>
           <t>7927646026</t>
         </is>
       </c>
-      <c r="B42" s="62" t="inlineStr">
+      <c r="B42" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C42" s="63" t="inlineStr">
+      <c r="C42" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00029/2026</t>
         </is>
       </c>
-      <c r="D42" s="62" t="inlineStr">
+      <c r="D42" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E42" s="62" t="n">
+      <c r="E42" s="57" t="n">
         <v>154</v>
       </c>
-      <c r="G42" s="62" t="inlineStr">
+      <c r="G42" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H42" s="63" t="inlineStr">
+      <c r="H42" s="58" t="inlineStr">
         <is>
           <t>Ponte Alta Tocantins</t>
         </is>
       </c>
-      <c r="I42" s="63" t="inlineStr">
+      <c r="I42" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3788,40 +3779,40 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="62" t="inlineStr">
+      <c r="A43" s="57" t="inlineStr">
         <is>
           <t>7931608059</t>
         </is>
       </c>
-      <c r="B43" s="62" t="inlineStr">
+      <c r="B43" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C43" s="63" t="inlineStr">
+      <c r="C43" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00040/2026</t>
         </is>
       </c>
-      <c r="D43" s="62" t="inlineStr">
+      <c r="D43" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E43" s="62" t="n">
+      <c r="E43" s="57" t="n">
         <v>133</v>
       </c>
-      <c r="G43" s="62" t="inlineStr">
+      <c r="G43" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H43" s="63" t="inlineStr">
+      <c r="H43" s="58" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I43" s="63" t="inlineStr">
+      <c r="I43" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3833,40 +3824,40 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="62" t="inlineStr">
+      <c r="A44" s="57" t="inlineStr">
         <is>
           <t>7908249152</t>
         </is>
       </c>
-      <c r="B44" s="62" t="inlineStr">
+      <c r="B44" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C44" s="63" t="inlineStr">
+      <c r="C44" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00038/2026</t>
         </is>
       </c>
-      <c r="D44" s="62" t="inlineStr">
+      <c r="D44" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E44" s="62" t="n">
+      <c r="E44" s="57" t="n">
         <v>133</v>
       </c>
-      <c r="G44" s="62" t="inlineStr">
+      <c r="G44" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H44" s="63" t="inlineStr">
+      <c r="H44" s="58" t="inlineStr">
         <is>
           <t>Santa Rosa Do Tocantins</t>
         </is>
       </c>
-      <c r="I44" s="63" t="inlineStr">
+      <c r="I44" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3878,40 +3869,40 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="62" t="inlineStr">
+      <c r="A45" s="57" t="inlineStr">
         <is>
           <t>7927396052</t>
         </is>
       </c>
-      <c r="B45" s="62" t="inlineStr">
+      <c r="B45" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C45" s="63" t="inlineStr">
+      <c r="C45" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00045/2026</t>
         </is>
       </c>
-      <c r="D45" s="62" t="inlineStr">
+      <c r="D45" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E45" s="62" t="n">
+      <c r="E45" s="57" t="n">
         <v>127</v>
       </c>
-      <c r="G45" s="62" t="inlineStr">
+      <c r="G45" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H45" s="63" t="inlineStr">
+      <c r="H45" s="58" t="inlineStr">
         <is>
           <t>Formoso Do Araguaia</t>
         </is>
       </c>
-      <c r="I45" s="63" t="inlineStr">
+      <c r="I45" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3923,40 +3914,40 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="62" t="inlineStr">
+      <c r="A46" s="57" t="inlineStr">
         <is>
           <t>7925871077</t>
         </is>
       </c>
-      <c r="B46" s="62" t="inlineStr">
+      <c r="B46" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C46" s="63" t="inlineStr">
+      <c r="C46" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00048/2026</t>
         </is>
       </c>
-      <c r="D46" s="62" t="inlineStr">
+      <c r="D46" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E46" s="62" t="n">
+      <c r="E46" s="57" t="n">
         <v>113</v>
       </c>
-      <c r="G46" s="62" t="inlineStr">
+      <c r="G46" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H46" s="63" t="inlineStr">
+      <c r="H46" s="58" t="inlineStr">
         <is>
           <t>Goiatins</t>
         </is>
       </c>
-      <c r="I46" s="63" t="inlineStr">
+      <c r="I46" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -3968,40 +3959,40 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="62" t="inlineStr">
+      <c r="A47" s="57" t="inlineStr">
         <is>
           <t>7953610256</t>
         </is>
       </c>
-      <c r="B47" s="62" t="inlineStr">
+      <c r="B47" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C47" s="63" t="inlineStr">
+      <c r="C47" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00050/2026</t>
         </is>
       </c>
-      <c r="D47" s="62" t="inlineStr">
+      <c r="D47" s="57" t="inlineStr">
         <is>
           <t>Muito Alto</t>
         </is>
       </c>
-      <c r="E47" s="62" t="n">
+      <c r="E47" s="57" t="n">
         <v>111</v>
       </c>
-      <c r="G47" s="62" t="inlineStr">
+      <c r="G47" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H47" s="63" t="inlineStr">
+      <c r="H47" s="58" t="inlineStr">
         <is>
           <t>Mateiros</t>
         </is>
       </c>
-      <c r="I47" s="63" t="inlineStr">
+      <c r="I47" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4013,40 +4004,40 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="62" t="inlineStr">
+      <c r="A48" s="57" t="inlineStr">
         <is>
           <t>7926442035</t>
         </is>
       </c>
-      <c r="B48" s="62" t="inlineStr">
+      <c r="B48" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C48" s="63" t="inlineStr">
+      <c r="C48" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00051/2026</t>
         </is>
       </c>
-      <c r="D48" s="62" t="inlineStr">
+      <c r="D48" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E48" s="62" t="n">
+      <c r="E48" s="57" t="n">
         <v>111</v>
       </c>
-      <c r="G48" s="62" t="inlineStr">
+      <c r="G48" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H48" s="63" t="inlineStr">
+      <c r="H48" s="58" t="inlineStr">
         <is>
           <t>Monte Do Carmo</t>
         </is>
       </c>
-      <c r="I48" s="63" t="inlineStr">
+      <c r="I48" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4058,40 +4049,40 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="62" t="inlineStr">
+      <c r="A49" s="57" t="inlineStr">
         <is>
           <t>7925744087</t>
         </is>
       </c>
-      <c r="B49" s="62" t="inlineStr">
+      <c r="B49" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C49" s="63" t="inlineStr">
+      <c r="C49" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00059/2026</t>
         </is>
       </c>
-      <c r="D49" s="62" t="inlineStr">
+      <c r="D49" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E49" s="62" t="n">
+      <c r="E49" s="57" t="n">
         <v>99</v>
       </c>
-      <c r="G49" s="62" t="inlineStr">
+      <c r="G49" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H49" s="63" t="inlineStr">
+      <c r="H49" s="58" t="inlineStr">
         <is>
           <t>Goianorte</t>
         </is>
       </c>
-      <c r="I49" s="63" t="inlineStr">
+      <c r="I49" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4103,40 +4094,40 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="62" t="inlineStr">
+      <c r="A50" s="57" t="inlineStr">
         <is>
           <t>7925733015</t>
         </is>
       </c>
-      <c r="B50" s="62" t="inlineStr">
+      <c r="B50" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C50" s="63" t="inlineStr">
+      <c r="C50" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00058/2026</t>
         </is>
       </c>
-      <c r="D50" s="62" t="inlineStr">
+      <c r="D50" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E50" s="62" t="n">
+      <c r="E50" s="57" t="n">
         <v>99</v>
       </c>
-      <c r="G50" s="62" t="inlineStr">
+      <c r="G50" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H50" s="63" t="inlineStr">
+      <c r="H50" s="58" t="inlineStr">
         <is>
           <t>Pedro Afonso</t>
         </is>
       </c>
-      <c r="I50" s="63" t="inlineStr">
+      <c r="I50" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4148,40 +4139,40 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="62" t="inlineStr">
+      <c r="A51" s="57" t="inlineStr">
         <is>
           <t>7901110084</t>
         </is>
       </c>
-      <c r="B51" s="62" t="inlineStr">
+      <c r="B51" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C51" s="63" t="inlineStr">
+      <c r="C51" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00061/2026</t>
         </is>
       </c>
-      <c r="D51" s="62" t="inlineStr">
+      <c r="D51" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E51" s="62" t="n">
+      <c r="E51" s="57" t="n">
         <v>98</v>
       </c>
-      <c r="G51" s="62" t="inlineStr">
+      <c r="G51" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H51" s="63" t="inlineStr">
+      <c r="H51" s="58" t="inlineStr">
         <is>
           <t>Divinopolis</t>
         </is>
       </c>
-      <c r="I51" s="63" t="inlineStr">
+      <c r="I51" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4193,40 +4184,40 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="62" t="inlineStr">
+      <c r="A52" s="57" t="inlineStr">
         <is>
           <t>7944559149</t>
         </is>
       </c>
-      <c r="B52" s="62" t="inlineStr">
+      <c r="B52" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C52" s="63" t="inlineStr">
+      <c r="C52" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00063/2026</t>
         </is>
       </c>
-      <c r="D52" s="62" t="inlineStr">
+      <c r="D52" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E52" s="62" t="n">
+      <c r="E52" s="57" t="n">
         <v>98</v>
       </c>
-      <c r="G52" s="62" t="inlineStr">
+      <c r="G52" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H52" s="63" t="inlineStr">
+      <c r="H52" s="58" t="inlineStr">
         <is>
           <t>Caseara</t>
         </is>
       </c>
-      <c r="I52" s="63" t="inlineStr">
+      <c r="I52" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4238,40 +4229,40 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="62" t="inlineStr">
+      <c r="A53" s="57" t="inlineStr">
         <is>
           <t>5800291035</t>
         </is>
       </c>
-      <c r="B53" s="62" t="inlineStr">
+      <c r="B53" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C53" s="63" t="inlineStr">
+      <c r="C53" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PO 00097/2026</t>
         </is>
       </c>
-      <c r="D53" s="62" t="inlineStr">
+      <c r="D53" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E53" s="62" t="n">
+      <c r="E53" s="57" t="n">
         <v>98</v>
       </c>
-      <c r="G53" s="62" t="inlineStr">
+      <c r="G53" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H53" s="63" t="inlineStr">
+      <c r="H53" s="58" t="inlineStr">
         <is>
           <t>Monte Do Carmo</t>
         </is>
       </c>
-      <c r="I53" s="64" t="inlineStr">
+      <c r="I53" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -4283,40 +4274,40 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="62" t="inlineStr">
+      <c r="A54" s="57" t="inlineStr">
         <is>
           <t>7919270014</t>
         </is>
       </c>
-      <c r="B54" s="62" t="inlineStr">
+      <c r="B54" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C54" s="63" t="inlineStr">
+      <c r="C54" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00074/2026</t>
         </is>
       </c>
-      <c r="D54" s="62" t="inlineStr">
+      <c r="D54" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E54" s="62" t="n">
+      <c r="E54" s="57" t="n">
         <v>82</v>
       </c>
-      <c r="G54" s="62" t="inlineStr">
+      <c r="G54" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H54" s="63" t="inlineStr">
+      <c r="H54" s="58" t="inlineStr">
         <is>
           <t>Pium</t>
         </is>
       </c>
-      <c r="I54" s="63" t="inlineStr">
+      <c r="I54" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4328,40 +4319,40 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="62" t="inlineStr">
+      <c r="A55" s="57" t="inlineStr">
         <is>
           <t>5801866013</t>
         </is>
       </c>
-      <c r="B55" s="62" t="inlineStr">
+      <c r="B55" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C55" s="63" t="inlineStr">
+      <c r="C55" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00077/2026</t>
         </is>
       </c>
-      <c r="D55" s="62" t="inlineStr">
+      <c r="D55" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E55" s="62" t="n">
+      <c r="E55" s="57" t="n">
         <v>79</v>
       </c>
-      <c r="G55" s="62" t="inlineStr">
+      <c r="G55" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H55" s="63" t="inlineStr">
+      <c r="H55" s="58" t="inlineStr">
         <is>
           <t>Paraiso Do Tocantins</t>
         </is>
       </c>
-      <c r="I55" s="63" t="inlineStr">
+      <c r="I55" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4373,40 +4364,40 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="62" t="inlineStr">
+      <c r="A56" s="57" t="inlineStr">
         <is>
           <t>7926089013</t>
         </is>
       </c>
-      <c r="B56" s="62" t="inlineStr">
+      <c r="B56" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C56" s="63" t="inlineStr">
+      <c r="C56" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00078/2026</t>
         </is>
       </c>
-      <c r="D56" s="62" t="inlineStr">
+      <c r="D56" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E56" s="62" t="n">
+      <c r="E56" s="57" t="n">
         <v>76</v>
       </c>
-      <c r="G56" s="62" t="inlineStr">
+      <c r="G56" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H56" s="63" t="inlineStr">
+      <c r="H56" s="58" t="inlineStr">
         <is>
           <t>Paraiso Do Tocantins</t>
         </is>
       </c>
-      <c r="I56" s="63" t="inlineStr">
+      <c r="I56" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4418,40 +4409,40 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="62" t="inlineStr">
+      <c r="A57" s="57" t="inlineStr">
         <is>
           <t>7900573047</t>
         </is>
       </c>
-      <c r="B57" s="62" t="inlineStr">
+      <c r="B57" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C57" s="63" t="inlineStr">
+      <c r="C57" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00080/2026</t>
         </is>
       </c>
-      <c r="D57" s="62" t="inlineStr">
+      <c r="D57" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E57" s="62" t="n">
+      <c r="E57" s="57" t="n">
         <v>75</v>
       </c>
-      <c r="G57" s="62" t="inlineStr">
+      <c r="G57" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H57" s="63" t="inlineStr">
+      <c r="H57" s="58" t="inlineStr">
         <is>
           <t>Figueiropolis</t>
         </is>
       </c>
-      <c r="I57" s="63" t="inlineStr">
+      <c r="I57" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4463,40 +4454,40 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="62" t="inlineStr">
+      <c r="A58" s="57" t="inlineStr">
         <is>
           <t>7927413001</t>
         </is>
       </c>
-      <c r="B58" s="62" t="inlineStr">
+      <c r="B58" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C58" s="63" t="inlineStr">
+      <c r="C58" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PO 00118/2026</t>
         </is>
       </c>
-      <c r="D58" s="62" t="inlineStr">
+      <c r="D58" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E58" s="62" t="n">
+      <c r="E58" s="57" t="n">
         <v>75</v>
       </c>
-      <c r="G58" s="62" t="inlineStr">
+      <c r="G58" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H58" s="63" t="inlineStr">
+      <c r="H58" s="58" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I58" s="64" t="inlineStr">
+      <c r="I58" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -4508,40 +4499,40 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="62" t="inlineStr">
+      <c r="A59" s="57" t="inlineStr">
         <is>
           <t>7908686014</t>
         </is>
       </c>
-      <c r="B59" s="62" t="inlineStr">
+      <c r="B59" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C59" s="63" t="inlineStr">
+      <c r="C59" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00086/2026</t>
         </is>
       </c>
-      <c r="D59" s="62" t="inlineStr">
+      <c r="D59" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E59" s="62" t="n">
+      <c r="E59" s="57" t="n">
         <v>74</v>
       </c>
-      <c r="G59" s="62" t="inlineStr">
+      <c r="G59" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H59" s="63" t="inlineStr">
+      <c r="H59" s="58" t="inlineStr">
         <is>
           <t>Pium</t>
         </is>
       </c>
-      <c r="I59" s="63" t="inlineStr">
+      <c r="I59" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4553,40 +4544,40 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="62" t="inlineStr">
+      <c r="A60" s="57" t="inlineStr">
         <is>
           <t>7900117013</t>
         </is>
       </c>
-      <c r="B60" s="62" t="inlineStr">
+      <c r="B60" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C60" s="63" t="inlineStr">
+      <c r="C60" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00084/2026</t>
         </is>
       </c>
-      <c r="D60" s="62" t="inlineStr">
+      <c r="D60" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E60" s="62" t="n">
+      <c r="E60" s="57" t="n">
         <v>74</v>
       </c>
-      <c r="G60" s="62" t="inlineStr">
+      <c r="G60" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H60" s="63" t="inlineStr">
+      <c r="H60" s="58" t="inlineStr">
         <is>
           <t>Paraiso Do Tocantins</t>
         </is>
       </c>
-      <c r="I60" s="63" t="inlineStr">
+      <c r="I60" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4598,40 +4589,40 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="62" t="inlineStr">
+      <c r="A61" s="57" t="inlineStr">
         <is>
           <t>7900453110</t>
         </is>
       </c>
-      <c r="B61" s="62" t="inlineStr">
+      <c r="B61" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C61" s="63" t="inlineStr">
+      <c r="C61" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00087/2026</t>
         </is>
       </c>
-      <c r="D61" s="62" t="inlineStr">
+      <c r="D61" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E61" s="62" t="n">
+      <c r="E61" s="57" t="n">
         <v>71</v>
       </c>
-      <c r="G61" s="62" t="inlineStr">
+      <c r="G61" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H61" s="63" t="inlineStr">
+      <c r="H61" s="58" t="inlineStr">
         <is>
           <t>Santa Rita Do Tocantins</t>
         </is>
       </c>
-      <c r="I61" s="63" t="inlineStr">
+      <c r="I61" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4643,40 +4634,40 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="62" t="inlineStr">
+      <c r="A62" s="57" t="inlineStr">
         <is>
           <t>5865120195</t>
         </is>
       </c>
-      <c r="B62" s="62" t="inlineStr">
+      <c r="B62" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C62" s="63" t="inlineStr">
+      <c r="C62" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-GR 00538/2026</t>
         </is>
       </c>
-      <c r="D62" s="62" t="inlineStr">
+      <c r="D62" s="57" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E62" s="62" t="n">
+      <c r="E62" s="57" t="n">
         <v>51</v>
       </c>
-      <c r="G62" s="62" t="inlineStr">
+      <c r="G62" s="57" t="inlineStr">
         <is>
           <t>COCM-N</t>
         </is>
       </c>
-      <c r="H62" s="63" t="inlineStr">
+      <c r="H62" s="58" t="inlineStr">
         <is>
           <t>Centenario</t>
         </is>
       </c>
-      <c r="I62" s="64" t="inlineStr">
+      <c r="I62" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -4688,40 +4679,40 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="62" t="inlineStr">
+      <c r="A63" s="57" t="inlineStr">
         <is>
           <t>5836786094</t>
         </is>
       </c>
-      <c r="B63" s="62" t="inlineStr">
+      <c r="B63" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C63" s="63" t="inlineStr">
+      <c r="C63" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00095/2026</t>
         </is>
       </c>
-      <c r="D63" s="62" t="inlineStr">
+      <c r="D63" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E63" s="62" t="n">
+      <c r="E63" s="57" t="n">
         <v>50</v>
       </c>
-      <c r="G63" s="62" t="inlineStr">
+      <c r="G63" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H63" s="63" t="inlineStr">
+      <c r="H63" s="58" t="inlineStr">
         <is>
           <t>Peixe</t>
         </is>
       </c>
-      <c r="I63" s="63" t="inlineStr">
+      <c r="I63" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4733,40 +4724,40 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="62" t="inlineStr">
+      <c r="A64" s="57" t="inlineStr">
         <is>
           <t>7900594026</t>
         </is>
       </c>
-      <c r="B64" s="62" t="inlineStr">
+      <c r="B64" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C64" s="63" t="inlineStr">
+      <c r="C64" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00113/2026</t>
         </is>
       </c>
-      <c r="D64" s="62" t="inlineStr">
+      <c r="D64" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E64" s="62" t="n">
+      <c r="E64" s="57" t="n">
         <v>27</v>
       </c>
-      <c r="G64" s="62" t="inlineStr">
+      <c r="G64" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H64" s="63" t="inlineStr">
+      <c r="H64" s="58" t="inlineStr">
         <is>
           <t>Ponte Alta Tocantins</t>
         </is>
       </c>
-      <c r="I64" s="63" t="inlineStr">
+      <c r="I64" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4778,40 +4769,40 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="62" t="inlineStr">
+      <c r="A65" s="57" t="inlineStr">
         <is>
           <t>7913662076</t>
         </is>
       </c>
-      <c r="B65" s="62" t="inlineStr">
+      <c r="B65" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C65" s="63" t="inlineStr">
+      <c r="C65" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00114/2026</t>
         </is>
       </c>
-      <c r="D65" s="62" t="inlineStr">
+      <c r="D65" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E65" s="62" t="n">
+      <c r="E65" s="57" t="n">
         <v>27</v>
       </c>
-      <c r="G65" s="62" t="inlineStr">
+      <c r="G65" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H65" s="63" t="inlineStr">
+      <c r="H65" s="58" t="inlineStr">
         <is>
           <t>Duere</t>
         </is>
       </c>
-      <c r="I65" s="63" t="inlineStr">
+      <c r="I65" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4823,40 +4814,40 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="62" t="inlineStr">
+      <c r="A66" s="57" t="inlineStr">
         <is>
           <t>5800859011</t>
         </is>
       </c>
-      <c r="B66" s="62" t="inlineStr">
+      <c r="B66" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C66" s="63" t="inlineStr">
+      <c r="C66" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00115/2026</t>
         </is>
       </c>
-      <c r="D66" s="62" t="inlineStr">
+      <c r="D66" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E66" s="62" t="n">
+      <c r="E66" s="57" t="n">
         <v>25</v>
       </c>
-      <c r="G66" s="62" t="inlineStr">
+      <c r="G66" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H66" s="63" t="inlineStr">
+      <c r="H66" s="58" t="inlineStr">
         <is>
           <t>Tupirama</t>
         </is>
       </c>
-      <c r="I66" s="63" t="inlineStr">
+      <c r="I66" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4868,40 +4859,40 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="62" t="inlineStr">
+      <c r="A67" s="57" t="inlineStr">
         <is>
           <t>5800090147</t>
         </is>
       </c>
-      <c r="B67" s="62" t="inlineStr">
+      <c r="B67" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C67" s="63" t="inlineStr">
+      <c r="C67" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00117/2026</t>
         </is>
       </c>
-      <c r="D67" s="62" t="inlineStr">
+      <c r="D67" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E67" s="62" t="n">
+      <c r="E67" s="57" t="n">
         <v>22</v>
       </c>
-      <c r="G67" s="62" t="inlineStr">
+      <c r="G67" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H67" s="63" t="inlineStr">
+      <c r="H67" s="58" t="inlineStr">
         <is>
           <t>Taipas Do Tocantins</t>
         </is>
       </c>
-      <c r="I67" s="63" t="inlineStr">
+      <c r="I67" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -4913,40 +4904,40 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="62" t="inlineStr">
+      <c r="A68" s="57" t="inlineStr">
         <is>
           <t>5856156091</t>
         </is>
       </c>
-      <c r="B68" s="62" t="inlineStr">
+      <c r="B68" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C68" s="63" t="inlineStr">
+      <c r="C68" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-DP 00403/2026</t>
         </is>
       </c>
-      <c r="D68" s="62" t="inlineStr">
+      <c r="D68" s="57" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E68" s="62" t="n">
+      <c r="E68" s="57" t="n">
         <v>8</v>
       </c>
-      <c r="G68" s="62" t="inlineStr">
+      <c r="G68" s="57" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H68" s="63" t="inlineStr">
+      <c r="H68" s="58" t="inlineStr">
         <is>
           <t>Almas</t>
         </is>
       </c>
-      <c r="I68" s="64" t="inlineStr">
+      <c r="I68" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -4958,40 +4949,40 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="62" t="inlineStr">
+      <c r="A69" s="57" t="inlineStr">
         <is>
           <t>5827102054</t>
         </is>
       </c>
-      <c r="B69" s="62" t="inlineStr">
+      <c r="B69" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C69" s="63" t="inlineStr">
+      <c r="C69" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PS 00289/2026</t>
         </is>
       </c>
-      <c r="D69" s="62" t="inlineStr">
+      <c r="D69" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E69" s="62" t="n">
+      <c r="E69" s="57" t="n">
         <v>8</v>
       </c>
-      <c r="G69" s="62" t="inlineStr">
+      <c r="G69" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H69" s="63" t="inlineStr">
+      <c r="H69" s="58" t="inlineStr">
         <is>
           <t>Pugmil</t>
         </is>
       </c>
-      <c r="I69" s="63" t="inlineStr">
+      <c r="I69" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5003,40 +4994,40 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="62" t="inlineStr">
+      <c r="A70" s="57" t="inlineStr">
         <is>
           <t>5846328094</t>
         </is>
       </c>
-      <c r="B70" s="62" t="inlineStr">
+      <c r="B70" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C70" s="63" t="inlineStr">
+      <c r="C70" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-GU 00687/2026</t>
         </is>
       </c>
-      <c r="D70" s="62" t="inlineStr">
+      <c r="D70" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E70" s="62" t="n">
+      <c r="E70" s="57" t="n">
         <v>8</v>
       </c>
-      <c r="G70" s="62" t="inlineStr">
+      <c r="G70" s="57" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H70" s="63" t="inlineStr">
+      <c r="H70" s="58" t="inlineStr">
         <is>
           <t>Peixe</t>
         </is>
       </c>
-      <c r="I70" s="64" t="inlineStr">
+      <c r="I70" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -5048,40 +5039,40 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="62" t="inlineStr">
+      <c r="A71" s="57" t="inlineStr">
         <is>
           <t>7942572059</t>
         </is>
       </c>
-      <c r="B71" s="62" t="inlineStr">
+      <c r="B71" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C71" s="63" t="inlineStr">
+      <c r="C71" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00427/2026</t>
         </is>
       </c>
-      <c r="D71" s="62" t="inlineStr">
+      <c r="D71" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E71" s="62" t="n">
+      <c r="E71" s="57" t="n">
         <v>8</v>
       </c>
-      <c r="G71" s="62" t="inlineStr">
+      <c r="G71" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H71" s="63" t="inlineStr">
+      <c r="H71" s="58" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I71" s="64" t="inlineStr">
+      <c r="I71" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -5093,40 +5084,40 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="62" t="inlineStr">
+      <c r="A72" s="57" t="inlineStr">
         <is>
           <t>7929376022</t>
         </is>
       </c>
-      <c r="B72" s="62" t="inlineStr">
+      <c r="B72" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C72" s="63" t="inlineStr">
+      <c r="C72" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00120/2026</t>
         </is>
       </c>
-      <c r="D72" s="62" t="inlineStr">
+      <c r="D72" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E72" s="62" t="n">
+      <c r="E72" s="57" t="n">
         <v>7</v>
       </c>
-      <c r="G72" s="62" t="inlineStr">
+      <c r="G72" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H72" s="63" t="inlineStr">
+      <c r="H72" s="58" t="inlineStr">
         <is>
           <t>Babaculandia</t>
         </is>
       </c>
-      <c r="I72" s="63" t="inlineStr">
+      <c r="I72" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5138,40 +5129,40 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="62" t="inlineStr">
+      <c r="A73" s="57" t="inlineStr">
         <is>
           <t>5800438116</t>
         </is>
       </c>
-      <c r="B73" s="62" t="inlineStr">
+      <c r="B73" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C73" s="63" t="inlineStr">
+      <c r="C73" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-DP 00404/2026</t>
         </is>
       </c>
-      <c r="D73" s="62" t="inlineStr">
+      <c r="D73" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E73" s="62" t="n">
+      <c r="E73" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="G73" s="62" t="inlineStr">
+      <c r="G73" s="57" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H73" s="63" t="inlineStr">
+      <c r="H73" s="58" t="inlineStr">
         <is>
           <t>Chapada Da Natividade</t>
         </is>
       </c>
-      <c r="I73" s="63" t="inlineStr">
+      <c r="I73" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5183,40 +5174,40 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="62" t="inlineStr">
+      <c r="A74" s="57" t="inlineStr">
         <is>
           <t>5803327001</t>
         </is>
       </c>
-      <c r="B74" s="62" t="inlineStr">
+      <c r="B74" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C74" s="63" t="inlineStr">
+      <c r="C74" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00434/2026</t>
         </is>
       </c>
-      <c r="D74" s="62" t="inlineStr">
+      <c r="D74" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E74" s="62" t="n">
+      <c r="E74" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="G74" s="62" t="inlineStr">
+      <c r="G74" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H74" s="63" t="inlineStr">
+      <c r="H74" s="58" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I74" s="64" t="inlineStr">
+      <c r="I74" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -5228,40 +5219,40 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="62" t="inlineStr">
+      <c r="A75" s="57" t="inlineStr">
         <is>
           <t>7933766059</t>
         </is>
       </c>
-      <c r="B75" s="62" t="inlineStr">
+      <c r="B75" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C75" s="63" t="inlineStr">
+      <c r="C75" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00431/2026</t>
         </is>
       </c>
-      <c r="D75" s="62" t="inlineStr">
+      <c r="D75" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E75" s="62" t="n">
+      <c r="E75" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="G75" s="62" t="inlineStr">
+      <c r="G75" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H75" s="63" t="inlineStr">
+      <c r="H75" s="58" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I75" s="63" t="inlineStr">
+      <c r="I75" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5273,40 +5264,40 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="62" t="inlineStr">
+      <c r="A76" s="57" t="inlineStr">
         <is>
           <t>7931610122</t>
         </is>
       </c>
-      <c r="B76" s="62" t="inlineStr">
+      <c r="B76" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C76" s="63" t="inlineStr">
+      <c r="C76" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00433/2026</t>
         </is>
       </c>
-      <c r="D76" s="62" t="inlineStr">
+      <c r="D76" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E76" s="62" t="n">
+      <c r="E76" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="G76" s="62" t="inlineStr">
+      <c r="G76" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H76" s="63" t="inlineStr">
+      <c r="H76" s="58" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="I76" s="63" t="inlineStr">
+      <c r="I76" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5318,40 +5309,40 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="62" t="inlineStr">
+      <c r="A77" s="57" t="inlineStr">
         <is>
           <t>7927169001</t>
         </is>
       </c>
-      <c r="B77" s="62" t="inlineStr">
+      <c r="B77" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C77" s="63" t="inlineStr">
+      <c r="C77" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PA 00432/2026</t>
         </is>
       </c>
-      <c r="D77" s="62" t="inlineStr">
+      <c r="D77" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E77" s="62" t="n">
+      <c r="E77" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="G77" s="62" t="inlineStr">
+      <c r="G77" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H77" s="63" t="inlineStr">
+      <c r="H77" s="58" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="I77" s="63" t="inlineStr">
+      <c r="I77" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5363,40 +5354,40 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="62" t="inlineStr">
+      <c r="A78" s="57" t="inlineStr">
         <is>
           <t>7933726256</t>
         </is>
       </c>
-      <c r="B78" s="62" t="inlineStr">
+      <c r="B78" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C78" s="63" t="inlineStr">
+      <c r="C78" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-PO 00181/2026</t>
         </is>
       </c>
-      <c r="D78" s="62" t="inlineStr">
+      <c r="D78" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E78" s="62" t="n">
+      <c r="E78" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="G78" s="62" t="inlineStr">
+      <c r="G78" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H78" s="63" t="inlineStr">
+      <c r="H78" s="58" t="inlineStr">
         <is>
           <t>Mateiros</t>
         </is>
       </c>
-      <c r="I78" s="63" t="inlineStr">
+      <c r="I78" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5408,40 +5399,40 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="62" t="inlineStr">
+      <c r="A79" s="57" t="inlineStr">
         <is>
           <t>7911120026</t>
         </is>
       </c>
-      <c r="B79" s="62" t="inlineStr">
+      <c r="B79" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C79" s="63" t="inlineStr">
+      <c r="C79" s="58" t="inlineStr">
         <is>
           <t>DG-RD-PO 00444/2026</t>
         </is>
       </c>
-      <c r="D79" s="62" t="inlineStr">
+      <c r="D79" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E79" s="62" t="n">
+      <c r="E79" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="G79" s="62" t="inlineStr">
+      <c r="G79" s="57" t="inlineStr">
         <is>
           <t>COCM-C</t>
         </is>
       </c>
-      <c r="H79" s="63" t="inlineStr">
+      <c r="H79" s="58" t="inlineStr">
         <is>
           <t>Ponte Alta Tocantins</t>
         </is>
       </c>
-      <c r="I79" s="64" t="inlineStr">
+      <c r="I79" s="59" t="inlineStr">
         <is>
           <t>Só no Mapeamento Criticidades</t>
         </is>
@@ -5453,40 +5444,40 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="62" t="inlineStr">
+      <c r="A80" s="57" t="inlineStr">
         <is>
           <t>7908705049</t>
         </is>
       </c>
-      <c r="B80" s="62" t="inlineStr">
+      <c r="B80" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C80" s="63" t="inlineStr">
+      <c r="C80" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-DP 00409/2026</t>
         </is>
       </c>
-      <c r="D80" s="62" t="inlineStr">
+      <c r="D80" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E80" s="62" t="n">
+      <c r="E80" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G80" s="62" t="inlineStr">
+      <c r="G80" s="57" t="inlineStr">
         <is>
           <t>COCM-S</t>
         </is>
       </c>
-      <c r="H80" s="63" t="inlineStr">
+      <c r="H80" s="58" t="inlineStr">
         <is>
           <t>Aurora Do Tocantins</t>
         </is>
       </c>
-      <c r="I80" s="63" t="inlineStr">
+      <c r="I80" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5498,40 +5489,40 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="62" t="inlineStr">
+      <c r="A81" s="57" t="inlineStr">
         <is>
           <t>7900230155</t>
         </is>
       </c>
-      <c r="B81" s="62" t="inlineStr">
+      <c r="B81" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C81" s="63" t="inlineStr">
+      <c r="C81" s="58" t="inlineStr">
         <is>
           <t>ETO-RD-GR 00685/2026</t>
         </is>
       </c>
-      <c r="D81" s="62" t="inlineStr">
+      <c r="D81" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E81" s="62" t="n">
+      <c r="E81" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G81" s="62" t="inlineStr">
+      <c r="G81" s="57" t="inlineStr">
         <is>
           <t>COCM-N</t>
         </is>
       </c>
-      <c r="H81" s="63" t="inlineStr">
+      <c r="H81" s="58" t="inlineStr">
         <is>
           <t>Palmeirante</t>
         </is>
       </c>
-      <c r="I81" s="63" t="inlineStr">
+      <c r="I81" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5543,40 +5534,40 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="62" t="inlineStr">
+      <c r="A82" s="57" t="inlineStr">
         <is>
           <t>7928564039</t>
         </is>
       </c>
-      <c r="B82" s="62" t="inlineStr">
+      <c r="B82" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C82" s="63" t="inlineStr">
+      <c r="C82" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00123/2026</t>
         </is>
       </c>
-      <c r="D82" s="62" t="inlineStr">
+      <c r="D82" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E82" s="62" t="n">
+      <c r="E82" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G82" s="62" t="inlineStr">
+      <c r="G82" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H82" s="63" t="inlineStr">
+      <c r="H82" s="58" t="inlineStr">
         <is>
           <t>Araguatins</t>
         </is>
       </c>
-      <c r="I82" s="63" t="inlineStr">
+      <c r="I82" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5588,40 +5579,40 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="62" t="inlineStr">
+      <c r="A83" s="57" t="inlineStr">
         <is>
           <t>7928241200</t>
         </is>
       </c>
-      <c r="B83" s="62" t="inlineStr">
+      <c r="B83" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C83" s="63" t="inlineStr">
+      <c r="C83" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00128/2026</t>
         </is>
       </c>
-      <c r="D83" s="62" t="inlineStr">
+      <c r="D83" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E83" s="62" t="n">
+      <c r="E83" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G83" s="62" t="inlineStr">
+      <c r="G83" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H83" s="63" t="inlineStr">
+      <c r="H83" s="58" t="inlineStr">
         <is>
           <t>Sao Salvador Do Tocantins</t>
         </is>
       </c>
-      <c r="I83" s="63" t="inlineStr">
+      <c r="I83" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5633,40 +5624,40 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="62" t="inlineStr">
+      <c r="A84" s="57" t="inlineStr">
         <is>
           <t>5856070091</t>
         </is>
       </c>
-      <c r="B84" s="62" t="inlineStr">
+      <c r="B84" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C84" s="63" t="inlineStr">
+      <c r="C84" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00130/2026</t>
         </is>
       </c>
-      <c r="D84" s="62" t="inlineStr">
+      <c r="D84" s="57" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E84" s="62" t="n">
+      <c r="E84" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G84" s="62" t="inlineStr">
+      <c r="G84" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H84" s="63" t="inlineStr">
+      <c r="H84" s="58" t="inlineStr">
         <is>
           <t>Almas</t>
         </is>
       </c>
-      <c r="I84" s="63" t="inlineStr">
+      <c r="I84" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5678,40 +5669,40 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="62" t="inlineStr">
+      <c r="A85" s="57" t="inlineStr">
         <is>
           <t>5850308009</t>
         </is>
       </c>
-      <c r="B85" s="62" t="inlineStr">
+      <c r="B85" s="57" t="inlineStr">
         <is>
           <t>RT (58)</t>
         </is>
       </c>
-      <c r="C85" s="63" t="inlineStr">
+      <c r="C85" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00127/2026</t>
         </is>
       </c>
-      <c r="D85" s="62" t="inlineStr">
+      <c r="D85" s="57" t="inlineStr">
         <is>
           <t>Baixo</t>
         </is>
       </c>
-      <c r="E85" s="62" t="n">
+      <c r="E85" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G85" s="62" t="inlineStr">
+      <c r="G85" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H85" s="63" t="inlineStr">
+      <c r="H85" s="58" t="inlineStr">
         <is>
           <t>Guarai</t>
         </is>
       </c>
-      <c r="I85" s="63" t="inlineStr">
+      <c r="I85" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5723,40 +5714,40 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="62" t="inlineStr">
+      <c r="A86" s="57" t="inlineStr">
         <is>
           <t>7937102148</t>
         </is>
       </c>
-      <c r="B86" s="62" t="inlineStr">
+      <c r="B86" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C86" s="63" t="inlineStr">
+      <c r="C86" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00129/2026</t>
         </is>
       </c>
-      <c r="D86" s="62" t="inlineStr">
+      <c r="D86" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E86" s="62" t="n">
+      <c r="E86" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G86" s="62" t="inlineStr">
+      <c r="G86" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H86" s="63" t="inlineStr">
+      <c r="H86" s="58" t="inlineStr">
         <is>
           <t>Sao Valerio Da Natividade</t>
         </is>
       </c>
-      <c r="I86" s="63" t="inlineStr">
+      <c r="I86" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5768,40 +5759,40 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="62" t="inlineStr">
+      <c r="A87" s="57" t="inlineStr">
         <is>
           <t>7923673004</t>
         </is>
       </c>
-      <c r="B87" s="62" t="inlineStr">
+      <c r="B87" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C87" s="63" t="inlineStr">
+      <c r="C87" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00124/2026</t>
         </is>
       </c>
-      <c r="D87" s="62" t="inlineStr">
+      <c r="D87" s="57" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="E87" s="62" t="n">
+      <c r="E87" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G87" s="62" t="inlineStr">
+      <c r="G87" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H87" s="63" t="inlineStr">
+      <c r="H87" s="58" t="inlineStr">
         <is>
           <t>Araguaina</t>
         </is>
       </c>
-      <c r="I87" s="63" t="inlineStr">
+      <c r="I87" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -5813,40 +5804,40 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="62" t="inlineStr">
+      <c r="A88" s="57" t="inlineStr">
         <is>
           <t>7900525015</t>
         </is>
       </c>
-      <c r="B88" s="62" t="inlineStr">
+      <c r="B88" s="57" t="inlineStr">
         <is>
           <t>RL (79)</t>
         </is>
       </c>
-      <c r="C88" s="63" t="inlineStr">
+      <c r="C88" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00125/2026</t>
         </is>
       </c>
-      <c r="D88" s="62" t="inlineStr">
+      <c r="D88" s="57" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="E88" s="62" t="n">
+      <c r="E88" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G88" s="62" t="inlineStr">
+      <c r="G88" s="57" t="inlineStr">
         <is>
           <t>COEP</t>
         </is>
       </c>
-      <c r="H88" s="63" t="inlineStr">
+      <c r="H88" s="58" t="inlineStr">
         <is>
           <t>Pedro Afonso</t>
         </is>
       </c>
-      <c r="I88" s="63" t="inlineStr">
+      <c r="I88" s="58" t="inlineStr">
         <is>
           <t>SIM (detalhamento)</t>
         </is>
@@ -14994,7 +14985,7 @@
       </c>
       <c r="J11" s="23" t="inlineStr">
         <is>
-          <t>COEP: não há compra de equipamento especial</t>
+          <t>CONFIRMADO NO SGM (print 08/07): cadeia ETO-TELE 00694/2025 &gt; ETO-COEP 00163/2025 (encerrada 29/06/2026, motivo NÃO É RESPONSABILIDADE DA ÁREA) &gt; repassada ETO-RD-PO 00180/2026 (COCM, pendente) e ETO-TELE 00975/2026 — sem compra COEP</t>
         </is>
       </c>
       <c r="K11" s="25" t="n">

</xml_diff>

<commit_message>
Inclui SS 00131/2026 (7947203070, Rio Sono) como equipamento completo
- Religador TAVRIDA 34,5 kV (Ajustes); decisão COEP de 08/07: compra do completo
- SS aberta após o congelamento — exceção anotada na Dinâmica e na linha
- Visão de SS atualizada: religadores 49 -> 50; total geral R$ 5.984.466,84

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBtNB8AfUGxQoc5b1rirVp
</commit_message>
<xml_diff>
--- a/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
+++ b/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
@@ -712,7 +712,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>⚠ DADOS CONGELADOS EM 07/07/2026 (D-1) — bases: SS pendentes posto COEP, OBRAS_EQ_ESPECIAL e ETO ATUALIZADA v10.</t>
+          <t>⚠ DADOS CONGELADOS EM 07/07/2026 (D-1) — bases: SS pendentes posto COEP, OBRAS_EQ_ESPECIAL e ETO ATUALIZADA v10. Exceção: SS 00131/2026 (7947203070), aberta em 08/07, incluída por instrução do gestor.</t>
         </is>
       </c>
     </row>
@@ -786,16 +786,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>2188151.77</v>
+        <v>2264397.97</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>592337.78</v>
+        <v>605547.12</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>2780489.55</v>
+        <v>2869945.09</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
@@ -871,16 +871,16 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>4477002.739999999</v>
+        <v>4553248.939999999</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>1418008.56</v>
+        <v>1431217.9</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>5895011.3</v>
+        <v>5984466.84</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10">
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="H13" s="11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I13" s="11" t="n">
         <v>18</v>
@@ -1005,16 +1005,16 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>1208112.37</v>
+        <v>1284358.57</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>321463.9000000001</v>
+        <v>334673.2400000001</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>1529576.27</v>
+        <v>1619031.81</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
@@ -1081,16 +1081,16 @@
         </is>
       </c>
       <c r="B18" s="19" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>2188151.77</v>
+        <v>2264397.97</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>592337.7800000001</v>
+        <v>605547.1200000001</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>2780489.55</v>
+        <v>2869945.09</v>
       </c>
     </row>
     <row r="20">
@@ -1187,16 +1187,16 @@
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C25" s="10" t="n">
-        <v>1187671.95</v>
+        <v>1263918.15</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>211404.38</v>
+        <v>224613.72</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>1399076.33</v>
+        <v>1488531.87</v>
       </c>
     </row>
     <row r="26">
@@ -1244,16 +1244,16 @@
         </is>
       </c>
       <c r="B28" s="19" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C28" s="8" t="n">
-        <v>2188151.77</v>
+        <v>2264397.97</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>592337.7799999999</v>
+        <v>605547.1199999999</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>2780489.549999999</v>
+        <v>2869945.09</v>
       </c>
     </row>
     <row r="30">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="61">
@@ -5926,16 +5926,16 @@
         </is>
       </c>
       <c r="B6" s="55" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6" s="55" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>2780489.550000001</v>
+        <v>2869945.090000001</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>59159.35212765959</v>
+        <v>59790.52270833335</v>
       </c>
     </row>
     <row r="7">
@@ -5983,13 +5983,13 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>5895011.300000001</v>
+        <v>5984466.840000001</v>
       </c>
       <c r="E9" s="17" t="n"/>
     </row>
@@ -12758,10 +12758,8 @@
           <t>Pendente (fora do posto)</t>
         </is>
       </c>
-      <c r="K103" s="23" t="inlineStr">
-        <is>
-          <t>(sem orçamento nesta base)</t>
-        </is>
+      <c r="K103" s="24" t="n">
+        <v>89455.53999999999</v>
       </c>
       <c r="L103" s="23" t="inlineStr">
         <is>
@@ -14400,7 +14398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -16950,27 +16948,27 @@
     <row r="41">
       <c r="A41" s="58" t="inlineStr">
         <is>
-          <t>ETO-COEP 00177/2025</t>
+          <t>ETO-COEP 00131/2026</t>
         </is>
       </c>
       <c r="B41" s="57" t="inlineStr">
         <is>
-          <t>7908705049</t>
+          <t>7947203070</t>
         </is>
       </c>
       <c r="C41" s="58" t="inlineStr">
         <is>
-          <t>Aurora do Tocantins</t>
+          <t>Rio Sono</t>
         </is>
       </c>
       <c r="D41" s="57" t="inlineStr">
         <is>
-          <t>COOPER F6</t>
+          <t>TAVRIDA</t>
         </is>
       </c>
       <c r="E41" s="57" t="inlineStr">
         <is>
-          <t>13,8</t>
+          <t>34,5</t>
         </is>
       </c>
       <c r="F41" s="58" t="inlineStr">
@@ -16980,58 +16978,58 @@
       </c>
       <c r="G41" s="23" t="inlineStr">
         <is>
-          <t>Religador completo</t>
+          <t>Religador completo (parte ativa + tanque) — decisão COEP 08/07</t>
         </is>
       </c>
       <c r="H41" s="24" t="n">
-        <v>55602.54</v>
+        <v>76246.2</v>
       </c>
       <c r="I41" s="24" t="n">
-        <v>11016.94</v>
+        <v>13209.34</v>
       </c>
       <c r="J41" s="23" t="inlineStr">
         <is>
-          <t>Fora da base de pendentes; EMD 511536, prev. 15/07</t>
+          <t>SS ABERTA EM 08/07 (após o congelamento de 07/07) — incluída por instrução do gestor. DMSL sem atualização de modelo/placa =&gt; compra do completo; COEP pergunta modelo da placa/código do material; TAVRIDA (Ajustes) sem sobressalente; ocorrência de 23/11/2025</t>
         </is>
       </c>
       <c r="K41" s="25" t="n">
-        <v>66619.48</v>
-      </c>
-      <c r="L41" s="26" t="inlineStr">
-        <is>
-          <t>Em execução (obra)</t>
+        <v>89455.53999999999</v>
+      </c>
+      <c r="L41" s="57" t="inlineStr">
+        <is>
+          <t>Só selecionado para Compra</t>
         </is>
       </c>
       <c r="M41" s="57" t="inlineStr">
         <is>
-          <t>0512600135</t>
-        </is>
-      </c>
-      <c r="N41" s="27" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N41" s="28" t="inlineStr">
+        <is>
+          <t>VERIFICAR</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="58" t="inlineStr">
         <is>
-          <t>ETO-COEP 00082/2026</t>
+          <t>ETO-COEP 00177/2025</t>
         </is>
       </c>
       <c r="B42" s="57" t="inlineStr">
         <is>
-          <t>7933766059</t>
+          <t>7908705049</t>
         </is>
       </c>
       <c r="C42" s="58" t="inlineStr">
         <is>
-          <t>Taquaralto</t>
+          <t>Aurora do Tocantins</t>
         </is>
       </c>
       <c r="D42" s="57" t="inlineStr">
         <is>
-          <t>NOJA RC10</t>
+          <t>COOPER F6</t>
         </is>
       </c>
       <c r="E42" s="57" t="inlineStr">
@@ -17041,168 +17039,168 @@
       </c>
       <c r="F42" s="58" t="inlineStr">
         <is>
-          <t>Parte ativa (Tanque)</t>
+          <t>Equipamento completo</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>Tanque (parte ativa)</t>
+          <t>Religador completo</t>
         </is>
       </c>
       <c r="H42" s="24" t="n">
-        <v>21785.72</v>
+        <v>55602.54</v>
       </c>
       <c r="I42" s="24" t="n">
         <v>11016.94</v>
       </c>
       <c r="J42" s="23" t="inlineStr">
         <is>
+          <t>Fora da base de pendentes; EMD 511536, prev. 15/07</t>
+        </is>
+      </c>
+      <c r="K42" s="25" t="n">
+        <v>66619.48</v>
+      </c>
+      <c r="L42" s="26" t="inlineStr">
+        <is>
+          <t>Em execução (obra)</t>
+        </is>
+      </c>
+      <c r="M42" s="57" t="inlineStr">
+        <is>
+          <t>0512600135</t>
+        </is>
+      </c>
+      <c r="N42" s="27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="58" t="inlineStr">
+        <is>
+          <t>ETO-COEP 00082/2026</t>
+        </is>
+      </c>
+      <c r="B43" s="57" t="inlineStr">
+        <is>
+          <t>7933766059</t>
+        </is>
+      </c>
+      <c r="C43" s="58" t="inlineStr">
+        <is>
+          <t>Taquaralto</t>
+        </is>
+      </c>
+      <c r="D43" s="57" t="inlineStr">
+        <is>
+          <t>NOJA RC10</t>
+        </is>
+      </c>
+      <c r="E43" s="57" t="inlineStr">
+        <is>
+          <t>13,8</t>
+        </is>
+      </c>
+      <c r="F43" s="58" t="inlineStr">
+        <is>
+          <t>Parte ativa (Tanque)</t>
+        </is>
+      </c>
+      <c r="G43" s="23" t="inlineStr">
+        <is>
+          <t>Tanque (parte ativa)</t>
+        </is>
+      </c>
+      <c r="H43" s="24" t="n">
+        <v>21785.72</v>
+      </c>
+      <c r="I43" s="24" t="n">
+        <v>11016.94</v>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
           <t>Obras cita SS 00211/2025 — adotada a mais recente (00082/2026); entrega concluída, substituição pendente</t>
         </is>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="K43" s="25" t="n">
         <v>32802.66</v>
       </c>
-      <c r="L42" s="26" t="inlineStr">
+      <c r="L43" s="26" t="inlineStr">
         <is>
           <t>Em execução (obra)</t>
         </is>
       </c>
-      <c r="M42" s="57" t="inlineStr">
+      <c r="M43" s="57" t="inlineStr">
         <is>
           <t>0112600424</t>
         </is>
       </c>
-      <c r="N42" s="27" t="inlineStr">
+      <c r="N43" s="27" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="46" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="46" t="inlineStr">
         <is>
           <t>ETO-COEP 00036/2026</t>
         </is>
       </c>
-      <c r="B43" s="45" t="inlineStr">
+      <c r="B44" s="45" t="inlineStr">
         <is>
           <t>7927169001</t>
         </is>
       </c>
-      <c r="C43" s="46" t="inlineStr">
+      <c r="C44" s="46" t="inlineStr">
         <is>
           <t>Porto Nacional</t>
         </is>
       </c>
-      <c r="D43" s="45" t="inlineStr">
+      <c r="D44" s="45" t="inlineStr">
         <is>
           <t>NOJA RC10</t>
         </is>
       </c>
-      <c r="E43" s="45" t="inlineStr">
+      <c r="E44" s="45" t="inlineStr">
         <is>
           <t>13,8</t>
         </is>
       </c>
-      <c r="F43" s="46" t="inlineStr">
+      <c r="F44" s="46" t="inlineStr">
         <is>
           <t>Equipamento completo</t>
         </is>
       </c>
-      <c r="G43" s="31" t="inlineStr">
+      <c r="G44" s="31" t="inlineStr">
         <is>
           <t>Religador completo — EM DÚVIDA (obras=completo x v1.5=tanque)</t>
         </is>
       </c>
-      <c r="H43" s="32" t="n">
+      <c r="H44" s="32" t="n">
         <v>55602.54</v>
       </c>
-      <c r="I43" s="32" t="n">
+      <c r="I44" s="32" t="n">
         <v>11016.94</v>
       </c>
-      <c r="J43" s="31" t="inlineStr">
+      <c r="J44" s="31" t="inlineStr">
         <is>
           <t>EM DÚVIDA =&gt; assumido EQUIPAMENTO COMPLETO (padrão do gestor). Modelo NOJA RC10 nos Ajustes (há peças) — AVALIAR na aba VERIFICAR</t>
         </is>
       </c>
-      <c r="K43" s="33" t="n">
+      <c r="K44" s="33" t="n">
         <v>66619.48</v>
       </c>
-      <c r="L43" s="45" t="inlineStr">
+      <c r="L44" s="45" t="inlineStr">
         <is>
           <t>Em execução (obra)</t>
         </is>
       </c>
-      <c r="M43" s="45" t="inlineStr">
+      <c r="M44" s="45" t="inlineStr">
         <is>
           <t>0112600425</t>
-        </is>
-      </c>
-      <c r="N43" s="28" t="inlineStr">
-        <is>
-          <t>VERIFICAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="58" t="inlineStr">
-        <is>
-          <t>ETO-COEP 00085/2026</t>
-        </is>
-      </c>
-      <c r="B44" s="57" t="inlineStr">
-        <is>
-          <t>7938137007</t>
-        </is>
-      </c>
-      <c r="C44" s="58" t="inlineStr">
-        <is>
-          <t>Miracema do Tocantins</t>
-        </is>
-      </c>
-      <c r="D44" s="57" t="inlineStr">
-        <is>
-          <t>SCHNEIDER ADVC</t>
-        </is>
-      </c>
-      <c r="E44" s="57" t="inlineStr">
-        <is>
-          <t>13,8</t>
-        </is>
-      </c>
-      <c r="F44" s="58" t="inlineStr">
-        <is>
-          <t>Componentes/Acessórios</t>
-        </is>
-      </c>
-      <c r="G44" s="23" t="inlineStr">
-        <is>
-          <t>Bateria + rádio + trafo/bucha fase A</t>
-        </is>
-      </c>
-      <c r="H44" s="24" t="n">
-        <v>14612.08</v>
-      </c>
-      <c r="I44" s="24" t="n">
-        <v>11016.94</v>
-      </c>
-      <c r="J44" s="23" t="inlineStr">
-        <is>
-          <t>Obras cita SS 00034/2026 — adotada a mais detalhada (00085/2026); rádio será testado/reaproveitado; 'entender sobre bucha da fase A'</t>
-        </is>
-      </c>
-      <c r="K44" s="25" t="n">
-        <v>25629.02</v>
-      </c>
-      <c r="L44" s="26" t="inlineStr">
-        <is>
-          <t>Em execução (obra)</t>
-        </is>
-      </c>
-      <c r="M44" s="57" t="inlineStr">
-        <is>
-          <t>0212600423</t>
         </is>
       </c>
       <c r="N44" s="28" t="inlineStr">
@@ -17214,52 +17212,52 @@
     <row r="45">
       <c r="A45" s="58" t="inlineStr">
         <is>
-          <t>ETO-COEP 00106/2025</t>
+          <t>ETO-COEP 00085/2026</t>
         </is>
       </c>
       <c r="B45" s="57" t="inlineStr">
         <is>
-          <t>7900230155</t>
+          <t>7938137007</t>
         </is>
       </c>
       <c r="C45" s="58" t="inlineStr">
         <is>
-          <t>Palmeirante</t>
+          <t>Miracema do Tocantins</t>
         </is>
       </c>
       <c r="D45" s="57" t="inlineStr">
         <is>
-          <t>COOPER F6</t>
+          <t>SCHNEIDER ADVC</t>
         </is>
       </c>
       <c r="E45" s="57" t="inlineStr">
         <is>
-          <t>34,5</t>
+          <t>13,8</t>
         </is>
       </c>
       <c r="F45" s="58" t="inlineStr">
         <is>
-          <t>Equipamento completo</t>
+          <t>Componentes/Acessórios</t>
         </is>
       </c>
       <c r="G45" s="23" t="inlineStr">
         <is>
-          <t>Tanque + controle NOJA enviado 07/07</t>
+          <t>Bateria + rádio + trafo/bucha fase A</t>
         </is>
       </c>
       <c r="H45" s="24" t="n">
-        <v>76246.2</v>
+        <v>14612.08</v>
       </c>
       <c r="I45" s="24" t="n">
-        <v>13209.34</v>
+        <v>11016.94</v>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>v1.5 (SS 00056/2025 — mesmo ano, adotada a mais recente 00106/2025) considerava só tanque; controle NOJA também enviado — custo de completo. Concluída parcialmente</t>
+          <t>Obras cita SS 00034/2026 — adotada a mais detalhada (00085/2026); rádio será testado/reaproveitado; 'entender sobre bucha da fase A'</t>
         </is>
       </c>
       <c r="K45" s="25" t="n">
-        <v>89455.53999999999</v>
+        <v>25629.02</v>
       </c>
       <c r="L45" s="26" t="inlineStr">
         <is>
@@ -17268,7 +17266,7 @@
       </c>
       <c r="M45" s="57" t="inlineStr">
         <is>
-          <t>0712600318</t>
+          <t>0212600423</t>
         </is>
       </c>
       <c r="N45" s="28" t="inlineStr">
@@ -17280,22 +17278,22 @@
     <row r="46">
       <c r="A46" s="58" t="inlineStr">
         <is>
-          <t>ETO-COEP 00181/2025</t>
+          <t>ETO-COEP 00106/2025</t>
         </is>
       </c>
       <c r="B46" s="57" t="inlineStr">
         <is>
-          <t>7943790134</t>
+          <t>7900230155</t>
         </is>
       </c>
       <c r="C46" s="58" t="inlineStr">
         <is>
-          <t>Esperantina</t>
+          <t>Palmeirante</t>
         </is>
       </c>
       <c r="D46" s="57" t="inlineStr">
         <is>
-          <t>NOJA RC10</t>
+          <t>COOPER F6</t>
         </is>
       </c>
       <c r="E46" s="57" t="inlineStr">
@@ -17305,58 +17303,58 @@
       </c>
       <c r="F46" s="58" t="inlineStr">
         <is>
-          <t>Parte ativa (Tanque)</t>
+          <t>Equipamento completo</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>Tanque (parte ativa)</t>
+          <t>Tanque + controle NOJA enviado 07/07</t>
         </is>
       </c>
       <c r="H46" s="24" t="n">
-        <v>38151.48</v>
+        <v>76246.2</v>
       </c>
       <c r="I46" s="24" t="n">
         <v>13209.34</v>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>CONCLUÍDA 06/06; obras: posto COEP 'Verificar' — confirmar baixa</t>
+          <t>v1.5 (SS 00056/2025 — mesmo ano, adotada a mais recente 00106/2025) considerava só tanque; controle NOJA também enviado — custo de completo. Concluída parcialmente</t>
         </is>
       </c>
       <c r="K46" s="25" t="n">
-        <v>51360.82000000001</v>
-      </c>
-      <c r="L46" s="57" t="inlineStr">
-        <is>
-          <t>Concluído</t>
+        <v>89455.53999999999</v>
+      </c>
+      <c r="L46" s="26" t="inlineStr">
+        <is>
+          <t>Em execução (obra)</t>
         </is>
       </c>
       <c r="M46" s="57" t="inlineStr">
         <is>
-          <t>0662600266</t>
-        </is>
-      </c>
-      <c r="N46" s="27" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>0712600318</t>
+        </is>
+      </c>
+      <c r="N46" s="28" t="inlineStr">
+        <is>
+          <t>VERIFICAR</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="58" t="inlineStr">
         <is>
-          <t>ETO-COEP 00178/2025</t>
+          <t>ETO-COEP 00181/2025</t>
         </is>
       </c>
       <c r="B47" s="57" t="inlineStr">
         <is>
-          <t>7900018004</t>
+          <t>7943790134</t>
         </is>
       </c>
       <c r="C47" s="58" t="inlineStr">
         <is>
-          <t>Araguaína</t>
+          <t>Esperantina</t>
         </is>
       </c>
       <c r="D47" s="57" t="inlineStr">
@@ -17371,27 +17369,27 @@
       </c>
       <c r="F47" s="58" t="inlineStr">
         <is>
-          <t>Equipamento completo</t>
+          <t>Parte ativa (Tanque)</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>Religador completo (Cooper→NOJA)</t>
+          <t>Tanque (parte ativa)</t>
         </is>
       </c>
       <c r="H47" s="24" t="n">
-        <v>76246.2</v>
+        <v>38151.48</v>
       </c>
       <c r="I47" s="24" t="n">
         <v>13209.34</v>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>CONCLUÍDA 27/05; tanque cooper retirado será usado no 7903112004</t>
+          <t>CONCLUÍDA 06/06; obras: posto COEP 'Verificar' — confirmar baixa</t>
         </is>
       </c>
       <c r="K47" s="25" t="n">
-        <v>89455.53999999999</v>
+        <v>51360.82000000001</v>
       </c>
       <c r="L47" s="57" t="inlineStr">
         <is>
@@ -17400,7 +17398,7 @@
       </c>
       <c r="M47" s="57" t="inlineStr">
         <is>
-          <t>0612600439</t>
+          <t>0662600266</t>
         </is>
       </c>
       <c r="N47" s="27" t="inlineStr">
@@ -17412,17 +17410,17 @@
     <row r="48">
       <c r="A48" s="58" t="inlineStr">
         <is>
-          <t>ETO-COEP 00083/2026</t>
+          <t>ETO-COEP 00178/2025</t>
         </is>
       </c>
       <c r="B48" s="57" t="inlineStr">
         <is>
-          <t>7931610122</t>
+          <t>7900018004</t>
         </is>
       </c>
       <c r="C48" s="58" t="inlineStr">
         <is>
-          <t>Palmas</t>
+          <t>Araguaína</t>
         </is>
       </c>
       <c r="D48" s="57" t="inlineStr">
@@ -17432,41 +17430,41 @@
       </c>
       <c r="E48" s="57" t="inlineStr">
         <is>
-          <t>13,8</t>
+          <t>34,5</t>
         </is>
       </c>
       <c r="F48" s="58" t="inlineStr">
         <is>
-          <t>Parte ativa (Tanque)</t>
+          <t>Equipamento completo</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
         <is>
-          <t>Tanque + antena</t>
+          <t>Religador completo (Cooper→NOJA)</t>
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>21785.72</v>
+        <v>76246.2</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>11016.94</v>
+        <v>13209.34</v>
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>Obras cita SS 00206/2025 — adotada a mais recente (00083/2026); substituição prev. 09/07</t>
+          <t>CONCLUÍDA 27/05; tanque cooper retirado será usado no 7903112004</t>
         </is>
       </c>
       <c r="K48" s="25" t="n">
-        <v>32802.66</v>
-      </c>
-      <c r="L48" s="26" t="inlineStr">
-        <is>
-          <t>Em execução (obra)</t>
+        <v>89455.53999999999</v>
+      </c>
+      <c r="L48" s="57" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="M48" s="57" t="inlineStr">
         <is>
-          <t>0112600383</t>
+          <t>0612600439</t>
         </is>
       </c>
       <c r="N48" s="27" t="inlineStr">
@@ -17478,17 +17476,17 @@
     <row r="49">
       <c r="A49" s="58" t="inlineStr">
         <is>
-          <t>ETO-COEP 00081/2026</t>
+          <t>ETO-COEP 00083/2026</t>
         </is>
       </c>
       <c r="B49" s="57" t="inlineStr">
         <is>
-          <t>7957620015</t>
+          <t>7931610122</t>
         </is>
       </c>
       <c r="C49" s="58" t="inlineStr">
         <is>
-          <t>Pedro Afonso</t>
+          <t>Palmas</t>
         </is>
       </c>
       <c r="D49" s="57" t="inlineStr">
@@ -17503,256 +17501,322 @@
       </c>
       <c r="F49" s="58" t="inlineStr">
         <is>
-          <t>Controle completo</t>
+          <t>Parte ativa (Tanque)</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
         <is>
-          <t>Rádio + antena + controle</t>
+          <t>Tanque + antena</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>33816.82</v>
+        <v>21785.72</v>
       </c>
       <c r="I49" s="24" t="n">
         <v>11016.94</v>
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
+          <t>Obras cita SS 00206/2025 — adotada a mais recente (00083/2026); substituição prev. 09/07</t>
+        </is>
+      </c>
+      <c r="K49" s="25" t="n">
+        <v>32802.66</v>
+      </c>
+      <c r="L49" s="26" t="inlineStr">
+        <is>
+          <t>Em execução (obra)</t>
+        </is>
+      </c>
+      <c r="M49" s="57" t="inlineStr">
+        <is>
+          <t>0112600383</t>
+        </is>
+      </c>
+      <c r="N49" s="27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="58" t="inlineStr">
+        <is>
+          <t>ETO-COEP 00081/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="57" t="inlineStr">
+        <is>
+          <t>7957620015</t>
+        </is>
+      </c>
+      <c r="C50" s="58" t="inlineStr">
+        <is>
+          <t>Pedro Afonso</t>
+        </is>
+      </c>
+      <c r="D50" s="57" t="inlineStr">
+        <is>
+          <t>NOJA RC10</t>
+        </is>
+      </c>
+      <c r="E50" s="57" t="inlineStr">
+        <is>
+          <t>13,8</t>
+        </is>
+      </c>
+      <c r="F50" s="58" t="inlineStr">
+        <is>
+          <t>Controle completo</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="inlineStr">
+        <is>
+          <t>Rádio + antena + controle</t>
+        </is>
+      </c>
+      <c r="H50" s="24" t="n">
+        <v>33816.82</v>
+      </c>
+      <c r="I50" s="24" t="n">
+        <v>11016.94</v>
+      </c>
+      <c r="J50" s="23" t="inlineStr">
+        <is>
           <t>Obras cita SS 00104/2025 — adotada a mais recente (00081/2026); CONCLUÍDA (22/05)</t>
         </is>
       </c>
-      <c r="K49" s="25" t="n">
+      <c r="K50" s="25" t="n">
         <v>44833.76</v>
       </c>
-      <c r="L49" s="57" t="inlineStr">
+      <c r="L50" s="57" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
-      <c r="M49" s="57" t="inlineStr">
+      <c r="M50" s="57" t="inlineStr">
         <is>
           <t>0712600316</t>
         </is>
       </c>
-      <c r="N49" s="27" t="inlineStr">
+      <c r="N50" s="27" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="46" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="46" t="inlineStr">
         <is>
           <t>ETO-COEP 00094/2025</t>
         </is>
       </c>
-      <c r="B50" s="45" t="inlineStr">
+      <c r="B51" s="45" t="inlineStr">
         <is>
           <t>7934698002</t>
         </is>
       </c>
-      <c r="C50" s="46" t="inlineStr">
+      <c r="C51" s="46" t="inlineStr">
         <is>
           <t>Tocantinópolis</t>
         </is>
       </c>
-      <c r="D50" s="45" t="inlineStr">
+      <c r="D51" s="45" t="inlineStr">
         <is>
           <t>NOJA RC10</t>
         </is>
       </c>
-      <c r="E50" s="45" t="inlineStr">
+      <c r="E51" s="45" t="inlineStr">
         <is>
           <t>13,8</t>
         </is>
       </c>
-      <c r="F50" s="46" t="inlineStr">
+      <c r="F51" s="46" t="inlineStr">
         <is>
           <t>Equipamento completo</t>
         </is>
       </c>
-      <c r="G50" s="31" t="inlineStr">
+      <c r="G51" s="31" t="inlineStr">
         <is>
           <t>Religador completo — EM DÚVIDA (obras=completo x v1.5=controle)</t>
         </is>
       </c>
-      <c r="H50" s="32" t="n">
+      <c r="H51" s="32" t="n">
         <v>55602.54</v>
       </c>
-      <c r="I50" s="32" t="n">
+      <c r="I51" s="32" t="n">
         <v>11016.94</v>
       </c>
-      <c r="J50" s="31" t="inlineStr">
+      <c r="J51" s="31" t="inlineStr">
         <is>
           <t>EM DÚVIDA =&gt; assumido EQUIPAMENTO COMPLETO (padrão do gestor). CONCLUÍDA 30/05 — confirmar o que foi aplicado; posto COEP 'Verificar'</t>
         </is>
       </c>
-      <c r="K50" s="33" t="n">
+      <c r="K51" s="33" t="n">
         <v>66619.48</v>
       </c>
-      <c r="L50" s="45" t="inlineStr">
+      <c r="L51" s="45" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
-      <c r="M50" s="45" t="inlineStr">
+      <c r="M51" s="45" t="inlineStr">
         <is>
           <t>0662600265</t>
         </is>
       </c>
-      <c r="N50" s="28" t="inlineStr">
+      <c r="N51" s="28" t="inlineStr">
         <is>
           <t>VERIFICAR</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="58" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="58" t="inlineStr">
         <is>
           <t>ETO-COEP 00151/2026</t>
         </is>
       </c>
-      <c r="B51" s="57" t="inlineStr">
+      <c r="B52" s="57" t="inlineStr">
         <is>
           <t>7955520116</t>
         </is>
       </c>
-      <c r="C51" s="58" t="inlineStr">
+      <c r="C52" s="58" t="inlineStr">
         <is>
           <t>Chapada da Natividade</t>
         </is>
       </c>
-      <c r="D51" s="57" t="inlineStr">
+      <c r="D52" s="57" t="inlineStr">
         <is>
           <t>NOJA RC10</t>
         </is>
       </c>
-      <c r="E51" s="57" t="inlineStr">
+      <c r="E52" s="57" t="inlineStr">
         <is>
           <t>34,5</t>
         </is>
       </c>
-      <c r="F51" s="58" t="inlineStr">
+      <c r="F52" s="58" t="inlineStr">
         <is>
           <t>Parte ativa (Tanque)</t>
         </is>
       </c>
-      <c r="G51" s="23" t="inlineStr">
+      <c r="G52" s="23" t="inlineStr">
         <is>
           <t>Tanque (parte ativa)</t>
         </is>
       </c>
-      <c r="H51" s="24" t="n">
+      <c r="H52" s="24" t="n">
         <v>38151.48</v>
       </c>
-      <c r="I51" s="24" t="n">
+      <c r="I52" s="24" t="n">
         <v>13209.34</v>
       </c>
-      <c r="J51" s="23" t="inlineStr">
+      <c r="J52" s="23" t="inlineStr">
         <is>
           <t>v1.5 cita SS 00149/2025 — adotada a mais recente (00151/2026); Requisitar=Não; EMD/entrega 'João verificar'</t>
         </is>
       </c>
-      <c r="K51" s="25" t="n">
+      <c r="K52" s="25" t="n">
         <v>51360.82000000001</v>
       </c>
-      <c r="L51" s="26" t="inlineStr">
+      <c r="L52" s="26" t="inlineStr">
         <is>
           <t>Em execução (obra)</t>
         </is>
       </c>
-      <c r="M51" s="57" t="inlineStr">
+      <c r="M52" s="57" t="inlineStr">
         <is>
           <t>0512600178</t>
         </is>
       </c>
-      <c r="N51" s="28" t="inlineStr">
+      <c r="N52" s="28" t="inlineStr">
         <is>
           <t>VERIFICAR</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="34" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="34" t="inlineStr">
         <is>
           <t>ETO-COEP 00108/2026</t>
         </is>
       </c>
-      <c r="B52" s="35" t="inlineStr">
+      <c r="B53" s="35" t="inlineStr">
         <is>
           <t>7933726256</t>
         </is>
       </c>
-      <c r="C52" s="34" t="inlineStr">
+      <c r="C53" s="34" t="inlineStr">
         <is>
           <t>Mateiros</t>
         </is>
       </c>
-      <c r="D52" s="35" t="inlineStr">
+      <c r="D53" s="35" t="inlineStr">
         <is>
           <t>NOJA RC10</t>
         </is>
       </c>
-      <c r="E52" s="35" t="inlineStr">
+      <c r="E53" s="35" t="inlineStr">
         <is>
           <t>34,5</t>
         </is>
       </c>
-      <c r="F52" s="34" t="inlineStr">
+      <c r="F53" s="34" t="inlineStr">
         <is>
           <t>Parte ativa (Tanque)</t>
         </is>
       </c>
-      <c r="G52" s="36" t="inlineStr">
+      <c r="G53" s="36" t="inlineStr">
         <is>
           <t>Tanque REAPROVEITADO (redirecionado de Santa Rita/7900453110)</t>
         </is>
       </c>
-      <c r="H52" s="37" t="n">
+      <c r="H53" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I52" s="37" t="n">
+      <c r="I53" s="37" t="n">
         <v>13209.34</v>
       </c>
-      <c r="J52" s="36" t="inlineStr">
+      <c r="J53" s="36" t="inlineStr">
         <is>
           <t>DISCUSSÃO COM MATHEUS ALVES — material R$ 0 (reaproveitamento); obras pede cancelar obra COCM</t>
         </is>
       </c>
-      <c r="K52" s="38" t="n">
+      <c r="K53" s="38" t="n">
         <v>13209.34</v>
       </c>
-      <c r="L52" s="35" t="inlineStr">
+      <c r="L53" s="35" t="inlineStr">
         <is>
           <t>Em execução (obra)</t>
         </is>
       </c>
-      <c r="M52" s="35" t="inlineStr">
+      <c r="M53" s="35" t="inlineStr">
         <is>
           <t>0312600351</t>
         </is>
       </c>
-      <c r="N52" s="28" t="inlineStr">
+      <c r="N53" s="28" t="inlineStr">
         <is>
           <t>VERIFICAR</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="G53" s="4" t="inlineStr">
+    <row r="54">
+      <c r="G54" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="H53" s="39" t="n">
-        <v>2188151.77</v>
-      </c>
-      <c r="I53" s="39" t="n">
-        <v>592337.78</v>
-      </c>
-      <c r="K53" s="39" t="n">
-        <v>2780489.55</v>
+      <c r="H54" s="39" t="n">
+        <v>2264397.97</v>
+      </c>
+      <c r="I54" s="39" t="n">
+        <v>605547.12</v>
+      </c>
+      <c r="K54" s="39" t="n">
+        <v>2869945.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Registra decisão: mandar o relé da SS 00124/2026 (7923673004)
Mesma SS já constava na base; confiança OK e decisão anotada na observação

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBtNB8AfUGxQoc5b1rirVp
</commit_message>
<xml_diff>
--- a/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
+++ b/ORCAMENTO_EQ_ESPECIAIS_V2.xlsx
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="61">
@@ -15922,7 +15922,7 @@
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>Relé prot. 50/51</t>
+          <t>Relé prot. 50/51 — MANDAR O RELÉ (decisão gestor 08/07)</t>
         </is>
       </c>
       <c r="H25" s="24" t="n">
@@ -15933,7 +15933,7 @@
       </c>
       <c r="J25" s="23" t="inlineStr">
         <is>
-          <t>Modelo em campo ARTECHE P500 — confirmar compatibilidade; SS 00057/2026 (v1.5) é duplicata — adotada a mais recente</t>
+          <t>DECISÃO DO GESTOR 08/07 (print SGM, mesma SS 00124/2026): mandar o relé (cód 625510). Modelo em campo ARTECHE P500; SS 00057/2026 (v1.5) é duplicata — adotada a mais recente</t>
         </is>
       </c>
       <c r="K25" s="25" t="n">
@@ -15949,9 +15949,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="N25" s="28" t="inlineStr">
-        <is>
-          <t>VERIFICAR</t>
+      <c r="N25" s="27" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>

</xml_diff>